<commit_message>
Se finaliza área de ficha tecnica
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sgc\storage\app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD444F5A-64AB-45F5-B04E-DF350792FC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7F08E0-2EA1-419D-8C98-3FB2F769BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B2495BF4-C32F-47F1-824B-FB221C6546E0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{28BFEBC5-EF34-42C7-846D-BB644F26337B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,33 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
+    <t>Cuenta Predial</t>
+  </si>
+  <si>
+    <t>Clave Catastral</t>
+  </si>
+  <si>
+    <t>Propietario</t>
+  </si>
+  <si>
+    <t>Ubicación del predio</t>
+  </si>
+  <si>
+    <t>Colindancias</t>
+  </si>
+  <si>
+    <t>Caracteristicas</t>
+  </si>
+  <si>
+    <t>Determinación del valor catastral</t>
+  </si>
+  <si>
+    <t>Imágenes</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
     <t>localidad</t>
   </si>
   <si>
@@ -72,9 +99,6 @@
     <t>departamento</t>
   </si>
   <si>
-    <t>Clave Catastral</t>
-  </si>
-  <si>
     <t>ap paterno</t>
   </si>
   <si>
@@ -96,9 +120,6 @@
     <t>sociedad</t>
   </si>
   <si>
-    <t>Propietario</t>
-  </si>
-  <si>
     <t>tipo asentamiento</t>
   </si>
   <si>
@@ -144,6 +165,9 @@
     <t>clave edificio</t>
   </si>
   <si>
+    <t>departamento edificio</t>
+  </si>
+  <si>
     <t>predio rustico antecedente</t>
   </si>
   <si>
@@ -153,15 +177,9 @@
     <t>longitud</t>
   </si>
   <si>
-    <t>Ubicación del predio</t>
-  </si>
-  <si>
     <t>colindancias</t>
   </si>
   <si>
-    <t>Colindancias</t>
-  </si>
-  <si>
     <t>clasificacion zona</t>
   </si>
   <si>
@@ -243,9 +261,6 @@
     <t>especiales</t>
   </si>
   <si>
-    <t>Caracteristicas</t>
-  </si>
-  <si>
     <t>terrenos</t>
   </si>
   <si>
@@ -264,13 +279,10 @@
     <t>uso 2</t>
   </si>
   <si>
-    <t xml:space="preserve">uso3 </t>
-  </si>
-  <si>
-    <t>ubicación manzana</t>
-  </si>
-  <si>
-    <t>Determinación del valor catastral</t>
+    <t xml:space="preserve">uso 3 </t>
+  </si>
+  <si>
+    <t>ubicacion manzana</t>
   </si>
   <si>
     <t>fachada</t>
@@ -294,26 +306,14 @@
     <t>representacion poligono</t>
   </si>
   <si>
-    <t>Imágenes</t>
-  </si>
-  <si>
-    <t>Observaciones</t>
-  </si>
-  <si>
     <t>observaciones</t>
-  </si>
-  <si>
-    <t>departamento edificio</t>
-  </si>
-  <si>
-    <t>Cuenta Predial</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -322,13 +322,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1" tint="0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -338,6 +348,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -361,13 +383,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -384,27 +400,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -719,22 +743,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{821B68B9-4210-4873-9DE3-137EF75E3827}">
-  <dimension ref="A1:CD2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7806A9-AE76-44CF-993F-CC0D365B724C}">
+  <dimension ref="A1:CD3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="82" max="82" width="15.44140625" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.88671875" style="7" customWidth="1"/>
+    <col min="40" max="40" width="16" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="26" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="50" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.5546875" style="7"/>
+    <col min="68" max="68" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="20.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="16" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:82" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+    <row r="1" spans="1:82" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
       <c r="E1" s="8" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
@@ -743,338 +816,342 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
       <c r="L1" s="8"/>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
+      <c r="AJ1" s="11"/>
+      <c r="AK1" s="11"/>
+      <c r="AL1" s="11"/>
+      <c r="AM1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="AN1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="AO1" s="12"/>
+      <c r="AP1" s="12"/>
+      <c r="AQ1" s="12"/>
+      <c r="AR1" s="12"/>
+      <c r="AS1" s="12"/>
+      <c r="AT1" s="12"/>
+      <c r="AU1" s="12"/>
+      <c r="AV1" s="12"/>
+      <c r="AW1" s="12"/>
+      <c r="AX1" s="12"/>
+      <c r="AY1" s="12"/>
+      <c r="AZ1" s="12"/>
+      <c r="BA1" s="12"/>
+      <c r="BB1" s="12"/>
+      <c r="BC1" s="12"/>
+      <c r="BD1" s="12"/>
+      <c r="BE1" s="12"/>
+      <c r="BF1" s="12"/>
+      <c r="BG1" s="12"/>
+      <c r="BH1" s="12"/>
+      <c r="BI1" s="12"/>
+      <c r="BJ1" s="12"/>
+      <c r="BK1" s="12"/>
+      <c r="BL1" s="12"/>
+      <c r="BM1" s="12"/>
+      <c r="BN1" s="12"/>
+      <c r="BO1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="BP1" s="10"/>
+      <c r="BQ1" s="10"/>
+      <c r="BR1" s="10"/>
+      <c r="BS1" s="10"/>
+      <c r="BT1" s="10"/>
+      <c r="BU1" s="10"/>
+      <c r="BV1" s="10"/>
+      <c r="BW1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="BX1" s="8"/>
+      <c r="BY1" s="8"/>
+      <c r="BZ1" s="8"/>
+      <c r="CA1" s="8"/>
+      <c r="CB1" s="8"/>
+      <c r="CC1" s="8"/>
+      <c r="CD1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:82" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="1" t="s">
+      <c r="M2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-      <c r="AF1" s="1"/>
-      <c r="AG1" s="1"/>
-      <c r="AH1" s="1"/>
-      <c r="AI1" s="1"/>
-      <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-      <c r="AM1" s="2" t="s">
+      <c r="AF2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AH2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AU2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AV2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="AX2" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AY2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AZ2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="BA2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="BB2" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="BC2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="BD2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="BE2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="BF2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="BG2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH2" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BI2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="AO1" s="3"/>
-      <c r="AP1" s="3"/>
-      <c r="AQ1" s="3"/>
-      <c r="AR1" s="3"/>
-      <c r="AS1" s="3"/>
-      <c r="AT1" s="3"/>
-      <c r="AU1" s="3"/>
-      <c r="AV1" s="3"/>
-      <c r="AW1" s="3"/>
-      <c r="AX1" s="3"/>
-      <c r="AY1" s="3"/>
-      <c r="AZ1" s="3"/>
-      <c r="BA1" s="3"/>
-      <c r="BB1" s="3"/>
-      <c r="BC1" s="3"/>
-      <c r="BD1" s="3"/>
-      <c r="BE1" s="3"/>
-      <c r="BF1" s="3"/>
-      <c r="BG1" s="3"/>
-      <c r="BH1" s="3"/>
-      <c r="BI1" s="3"/>
-      <c r="BJ1" s="3"/>
-      <c r="BK1" s="3"/>
-      <c r="BL1" s="3"/>
-      <c r="BM1" s="3"/>
-      <c r="BN1" s="3"/>
-      <c r="BO1" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="BK2" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="BL2" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="BM2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="BN2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="BO2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="BP2" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="BQ2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="BR2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="BP1" s="4"/>
-      <c r="BQ1" s="4"/>
-      <c r="BR1" s="4"/>
-      <c r="BS1" s="4"/>
-      <c r="BT1" s="4"/>
-      <c r="BU1" s="4"/>
-      <c r="BV1" s="4"/>
-      <c r="BW1" s="5" t="s">
+      <c r="BS2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="BT2" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="BU2" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="BV2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="BW2" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="BX2" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="BY2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="BZ2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="BX1" s="5"/>
-      <c r="BY1" s="5"/>
-      <c r="BZ1" s="5"/>
-      <c r="CA1" s="5"/>
-      <c r="CB1" s="5"/>
-      <c r="CC1" s="5"/>
-      <c r="CD1" s="6" t="s">
+      <c r="CA2" s="4" t="s">
         <v>87</v>
       </c>
+      <c r="CB2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="CC2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="CD2" s="4" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="2" spans="1:82" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" t="s">
-        <v>14</v>
-      </c>
-      <c r="O2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>17</v>
-      </c>
-      <c r="R2" t="s">
-        <v>18</v>
-      </c>
-      <c r="S2" t="s">
-        <v>19</v>
-      </c>
-      <c r="T2" t="s">
-        <v>21</v>
-      </c>
-      <c r="U2" t="s">
-        <v>22</v>
-      </c>
-      <c r="V2" t="s">
-        <v>23</v>
-      </c>
-      <c r="W2" t="s">
-        <v>24</v>
-      </c>
-      <c r="X2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>26</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>28</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>38</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>47</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>49</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>54</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>55</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>56</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>57</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>58</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>59</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>60</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>61</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>62</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>63</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>64</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>65</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>66</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>68</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>70</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>71</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>72</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>73</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>74</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>75</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>76</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>77</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>79</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>80</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>81</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>82</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>83</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>84</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>88</v>
-      </c>
+    <row r="3" spans="1:82" x14ac:dyDescent="0.3">
+      <c r="BS3" s="7"/>
+      <c r="BV3" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Ajustes en constantesm asignacion de cuenta predial, ficha tecnica
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sgc\storage\app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7F08E0-2EA1-419D-8C98-3FB2F769BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A72C4D4-1D41-4E94-901C-118B8DBF81F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{28BFEBC5-EF34-42C7-846D-BB644F26337B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="416">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -307,6 +308,981 @@
   </si>
   <si>
     <t>observaciones</t>
+  </si>
+  <si>
+    <t>FISICA</t>
+  </si>
+  <si>
+    <t>FIDUCIARIO</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>AEROPUERTO</t>
+  </si>
+  <si>
+    <t>CIRCUITO</t>
+  </si>
+  <si>
+    <t>INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>DOS NIVELES (MEDIA)</t>
+  </si>
+  <si>
+    <t>NO APLICA</t>
+  </si>
+  <si>
+    <t>ASILO</t>
+  </si>
+  <si>
+    <t>ESQUINA</t>
+  </si>
+  <si>
+    <t>si no</t>
+  </si>
+  <si>
+    <t>tipo construccion dominant</t>
+  </si>
+  <si>
+    <t>uso</t>
+  </si>
+  <si>
+    <t>MORAL</t>
+  </si>
+  <si>
+    <t>NUDO-PROPIETARIO</t>
+  </si>
+  <si>
+    <t>USUFRUCTUARIO</t>
+  </si>
+  <si>
+    <t>JUBILADO O PENSIONADO</t>
+  </si>
+  <si>
+    <t>FIDECOMITENTE</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>AMPLIACIÓN</t>
+  </si>
+  <si>
+    <t>BARRIO</t>
+  </si>
+  <si>
+    <t>CANTON</t>
+  </si>
+  <si>
+    <t>CIUDAD</t>
+  </si>
+  <si>
+    <t>CIUDAD INSDUSTRIAL</t>
+  </si>
+  <si>
+    <t>COLONIA</t>
+  </si>
+  <si>
+    <t>CONDOMINIO</t>
+  </si>
+  <si>
+    <t>CONJUNTO HABITACIONAL</t>
+  </si>
+  <si>
+    <t>CORREDOR INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>COTO</t>
+  </si>
+  <si>
+    <t>CUARTEL</t>
+  </si>
+  <si>
+    <t>EJIDO</t>
+  </si>
+  <si>
+    <t>EX-EJIDO</t>
+  </si>
+  <si>
+    <t>EXHACIENDA</t>
+  </si>
+  <si>
+    <t>FRACCIÓN</t>
+  </si>
+  <si>
+    <t>FRACCIONAMIENTO</t>
+  </si>
+  <si>
+    <t>GRANJA</t>
+  </si>
+  <si>
+    <t>HACIENDA</t>
+  </si>
+  <si>
+    <t>INGENIO</t>
+  </si>
+  <si>
+    <t>MANZANA</t>
+  </si>
+  <si>
+    <t>PARAJE</t>
+  </si>
+  <si>
+    <t>PARQUE INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>POBLADO</t>
+  </si>
+  <si>
+    <t>PRIVADA</t>
+  </si>
+  <si>
+    <t>PROLONGACIÓN</t>
+  </si>
+  <si>
+    <t>PUEBLO</t>
+  </si>
+  <si>
+    <t>PUERTO</t>
+  </si>
+  <si>
+    <t>RANCHERIA</t>
+  </si>
+  <si>
+    <t>RANCHO</t>
+  </si>
+  <si>
+    <t>REGIÓN</t>
+  </si>
+  <si>
+    <t>RESIDENCIAL</t>
+  </si>
+  <si>
+    <t>RINCONADA</t>
+  </si>
+  <si>
+    <t>SECCIÓN</t>
+  </si>
+  <si>
+    <t>SECTOR</t>
+  </si>
+  <si>
+    <t>SUPERMANZANA</t>
+  </si>
+  <si>
+    <t>TENENCIA</t>
+  </si>
+  <si>
+    <t>UNIDAD</t>
+  </si>
+  <si>
+    <t>UNIDAD HABITACIONAL</t>
+  </si>
+  <si>
+    <t>VILLA</t>
+  </si>
+  <si>
+    <t>ZONA FEDERAL</t>
+  </si>
+  <si>
+    <t>ZONA INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>ZONA MILITAR</t>
+  </si>
+  <si>
+    <t>ZONA NAVAL</t>
+  </si>
+  <si>
+    <t>ANDADOR</t>
+  </si>
+  <si>
+    <t>ARROYO O CANAL</t>
+  </si>
+  <si>
+    <t>AVENIDA</t>
+  </si>
+  <si>
+    <t>BOULEVARD</t>
+  </si>
+  <si>
+    <t>BRECHA</t>
+  </si>
+  <si>
+    <t>CALLE</t>
+  </si>
+  <si>
+    <t>CALLEJÓN</t>
+  </si>
+  <si>
+    <t>CALZADA</t>
+  </si>
+  <si>
+    <t>CAMINO</t>
+  </si>
+  <si>
+    <t>CAMINO REAL</t>
+  </si>
+  <si>
+    <t>CARRETERA</t>
+  </si>
+  <si>
+    <t>CERRADA</t>
+  </si>
+  <si>
+    <t>CIRCUNVALACIÓN</t>
+  </si>
+  <si>
+    <t>CONTINUACIÓN</t>
+  </si>
+  <si>
+    <t>CORREDOR</t>
+  </si>
+  <si>
+    <t>DIAGONAL</t>
+  </si>
+  <si>
+    <t>EJE VIAL</t>
+  </si>
+  <si>
+    <t>PASAJE</t>
+  </si>
+  <si>
+    <t>PEATONAL</t>
+  </si>
+  <si>
+    <t>PERIFÉRICO</t>
+  </si>
+  <si>
+    <t>PLAZA</t>
+  </si>
+  <si>
+    <t>PORTAL</t>
+  </si>
+  <si>
+    <t>RETORNO</t>
+  </si>
+  <si>
+    <t>SERVIDUMBRE DE PASO</t>
+  </si>
+  <si>
+    <t>VIADUCTO</t>
+  </si>
+  <si>
+    <t>HAB. DEN. SUBURBANA MENOR 50 HAB POR HA</t>
+  </si>
+  <si>
+    <t>HAB. DEN. BAJA 51 - 150 HAB POR HA</t>
+  </si>
+  <si>
+    <t>HAB. DEN. MEDIA 151 - 300 HAB POR HA</t>
+  </si>
+  <si>
+    <t>HAB. DEN. ALTA 301 - 500 HAB POR HA</t>
+  </si>
+  <si>
+    <t>HAB. DEN. MEDIA SE Y CO,300 HAB POR HA</t>
+  </si>
+  <si>
+    <t>HAB. DEN. MEDIA CO IN Y SE,300 HABPORHA</t>
+  </si>
+  <si>
+    <t>SUBCENTRO URBANO HASTA 120 VIV POR HA</t>
+  </si>
+  <si>
+    <t>CENTRO URBANO HASTA 120 VIV POR HA</t>
+  </si>
+  <si>
+    <t>CENTRO METROP. HASTA 72 VIV POR HA</t>
+  </si>
+  <si>
+    <t>ZONA DE MONUMENTOS</t>
+  </si>
+  <si>
+    <t>ZONA DE TRANSICIÓN</t>
+  </si>
+  <si>
+    <t>ÁREAS VERDES YO EQUIPAMIENTO</t>
+  </si>
+  <si>
+    <t>PARQUE URBANO ECOLÓGICO</t>
+  </si>
+  <si>
+    <t>EQUIPAMIENTO</t>
+  </si>
+  <si>
+    <t>INFRAESTRUCTURA</t>
+  </si>
+  <si>
+    <t>VIALIDAD Y DERECHO DE PASO</t>
+  </si>
+  <si>
+    <t>PROTECCIÓN ESPECIAL</t>
+  </si>
+  <si>
+    <t>PROTECCIÓN ECOLÓGICA ESPECIAL</t>
+  </si>
+  <si>
+    <t>ÁREA NATURAL PROTEGIDA (DECRETADA)</t>
+  </si>
+  <si>
+    <t>ZONA DE RESTAURACIÓN Y PROT. AMBIENTAL</t>
+  </si>
+  <si>
+    <t>PROTECCIÓN AGROPECUARIA</t>
+  </si>
+  <si>
+    <t>PROTECCIÓN USOS AGRICOLAS</t>
+  </si>
+  <si>
+    <t>PROTECCIÓN USOS PECUARIOS</t>
+  </si>
+  <si>
+    <t>COMERCIAL Y HABITACIONAL</t>
+  </si>
+  <si>
+    <t>UN NIVEL (ECONOMICA)</t>
+  </si>
+  <si>
+    <t>UN NIVEL (IND. LIGERA)</t>
+  </si>
+  <si>
+    <t>UN NIVEL  (IND. MEDIA)</t>
+  </si>
+  <si>
+    <t>UN NIVEL  (PESADA)</t>
+  </si>
+  <si>
+    <t>DOS NIVELES (MEDIA -SUPERIOR)</t>
+  </si>
+  <si>
+    <t>DOS  NIVELES  (SUPERIOR)</t>
+  </si>
+  <si>
+    <t>UNO Y DOS NIVELES  (ECONOMICA - MEDIA)</t>
+  </si>
+  <si>
+    <t>UNO Y DOS NIVELES  (IND. LIGERA Y MEDIA)</t>
+  </si>
+  <si>
+    <t>UNO Y DOS NIVELES  (IND. MEDIA - PESADA)</t>
+  </si>
+  <si>
+    <t>DOS Y TRES NIVELES (MEDIA - SUPERIOR)</t>
+  </si>
+  <si>
+    <t>MAMPOSTERIA</t>
+  </si>
+  <si>
+    <t>ZAPATA ASILADA</t>
+  </si>
+  <si>
+    <t>ZAPATAS CORRIDAS</t>
+  </si>
+  <si>
+    <t>LOSA DE CIMENTACION</t>
+  </si>
+  <si>
+    <t>COLUMNAS CANTERA O MADERA</t>
+  </si>
+  <si>
+    <t>TRABES, CASTILLOS, CADENA DE CERRAMIENTO</t>
+  </si>
+  <si>
+    <t>C. CONCRE., TRABES, CAST. Y C. DE CERRAM</t>
+  </si>
+  <si>
+    <t>C. METALI., TRABES, CAST. Y C. DE CERRAM</t>
+  </si>
+  <si>
+    <t>MUROS DE CARGA DE CONCRETO ARMADO</t>
+  </si>
+  <si>
+    <t>MULTIPANEL</t>
+  </si>
+  <si>
+    <t>MADERA Y ADOBE</t>
+  </si>
+  <si>
+    <t>PIEDRA O ADOBE</t>
+  </si>
+  <si>
+    <t>TABIQUE Y/O TABICON</t>
+  </si>
+  <si>
+    <t>TABIQUE Y CONCRETO</t>
+  </si>
+  <si>
+    <t>COCRETO ARMADO</t>
+  </si>
+  <si>
+    <t>BOVEDA  CATALANA</t>
+  </si>
+  <si>
+    <t>MADERA</t>
+  </si>
+  <si>
+    <t>LOSA RETICULAR</t>
+  </si>
+  <si>
+    <t>LOSA DE CONCRETO  REFORZADO</t>
+  </si>
+  <si>
+    <t>ESTRUCTURA METALICA O MIXTA</t>
+  </si>
+  <si>
+    <t>ARMADURAS DE MONTEN O ANGULOS SENCILLOS</t>
+  </si>
+  <si>
+    <t>ARMADURAS METALICAS DE PERALTE REGULAR</t>
+  </si>
+  <si>
+    <t>ARMADURAS  METALICAS DE GRAN PERALTE</t>
+  </si>
+  <si>
+    <t>TRIDILOSA</t>
+  </si>
+  <si>
+    <t>TEJA</t>
+  </si>
+  <si>
+    <t>LAMINA DE CARTON</t>
+  </si>
+  <si>
+    <t>LAMINA ACRILICA</t>
+  </si>
+  <si>
+    <t>LAMINA GALVANIZADA</t>
+  </si>
+  <si>
+    <t>LAMINA DE ASBESTO-CEMENTO</t>
+  </si>
+  <si>
+    <t>LAMINA DE CARTON-ASBESTO-CEMENTO</t>
+  </si>
+  <si>
+    <t>MANTA DE CIELO</t>
+  </si>
+  <si>
+    <t>MEZCLA DE MORTERO</t>
+  </si>
+  <si>
+    <t>YESO Y/O PASTA</t>
+  </si>
+  <si>
+    <t>FLASO PLAFON</t>
+  </si>
+  <si>
+    <t>TABLAROCA</t>
+  </si>
+  <si>
+    <t>SENCILLOS 3MM, LISO Y/O CHINO</t>
+  </si>
+  <si>
+    <t>SEMI DOBLE 6MM LISO Y/O CHINO O COLOR</t>
+  </si>
+  <si>
+    <t>FILTRASOL DE VARIOS ESPESORES</t>
+  </si>
+  <si>
+    <t>EMPLOMADO</t>
+  </si>
+  <si>
+    <t>TEMPLADO</t>
+  </si>
+  <si>
+    <t>VITRALES</t>
+  </si>
+  <si>
+    <t>MADERAS</t>
+  </si>
+  <si>
+    <t>AZULEJO</t>
+  </si>
+  <si>
+    <t>CERAMICA</t>
+  </si>
+  <si>
+    <t>CEMENTO</t>
+  </si>
+  <si>
+    <t>MOSAICO</t>
+  </si>
+  <si>
+    <t>LOSETA DE BARRO</t>
+  </si>
+  <si>
+    <t>PARQUET</t>
+  </si>
+  <si>
+    <t>DUELA</t>
+  </si>
+  <si>
+    <t>FIERRO FORJADO</t>
+  </si>
+  <si>
+    <t>ESTRUCTURAL</t>
+  </si>
+  <si>
+    <t>TUBULAR</t>
+  </si>
+  <si>
+    <t>ALUMINIO DE VARIOS CALIBRES</t>
+  </si>
+  <si>
+    <t>A LA CAL</t>
+  </si>
+  <si>
+    <t>VINILICA</t>
+  </si>
+  <si>
+    <t>ESMALTE</t>
+  </si>
+  <si>
+    <t>MADERA ECONOMICA</t>
+  </si>
+  <si>
+    <t>MADERA DE MEDIANA CALIDAD</t>
+  </si>
+  <si>
+    <t>MADERAS FINAS</t>
+  </si>
+  <si>
+    <t>ESTUCO</t>
+  </si>
+  <si>
+    <t>BARRO</t>
+  </si>
+  <si>
+    <t>YESO</t>
+  </si>
+  <si>
+    <t>PASTAS</t>
+  </si>
+  <si>
+    <t>PAPEL TAPIZ</t>
+  </si>
+  <si>
+    <t>ALFOMBRA</t>
+  </si>
+  <si>
+    <t>PIEDRA</t>
+  </si>
+  <si>
+    <t>GALVANIZADA</t>
+  </si>
+  <si>
+    <t>GALVANIZADA, COBRE</t>
+  </si>
+  <si>
+    <t>COBRE Y/O PVC</t>
+  </si>
+  <si>
+    <t>ALBAÑAL DE CEMENTO</t>
+  </si>
+  <si>
+    <t>ALBAÑAL FORJADO</t>
+  </si>
+  <si>
+    <t>PVC VARIOS DIAMETROS</t>
+  </si>
+  <si>
+    <t>VISIBLES</t>
+  </si>
+  <si>
+    <t>OCULTA</t>
+  </si>
+  <si>
+    <t>COBRE</t>
+  </si>
+  <si>
+    <t>GAS ESTACIONARIO</t>
+  </si>
+  <si>
+    <t>INTERFON</t>
+  </si>
+  <si>
+    <t>CIRCUITO CERRADO DE TV</t>
+  </si>
+  <si>
+    <t>AGENCIA DE AUTOS</t>
+  </si>
+  <si>
+    <t>AGENCIA DE VIAJES</t>
+  </si>
+  <si>
+    <t>AGOSTADERO</t>
+  </si>
+  <si>
+    <t>AGRICOLA</t>
+  </si>
+  <si>
+    <t>AGROPECUARIO</t>
+  </si>
+  <si>
+    <t>ALBERCA</t>
+  </si>
+  <si>
+    <t>ALBERGUE</t>
+  </si>
+  <si>
+    <t>APARTAMENTO</t>
+  </si>
+  <si>
+    <t>ASISTENCIA PUBLICA</t>
+  </si>
+  <si>
+    <t>AUTO LAVADO</t>
+  </si>
+  <si>
+    <t>BALDIO</t>
+  </si>
+  <si>
+    <t>BALNEARIO</t>
+  </si>
+  <si>
+    <t>BANCOS</t>
+  </si>
+  <si>
+    <t>BAÑOS</t>
+  </si>
+  <si>
+    <t>BASCULA</t>
+  </si>
+  <si>
+    <t>BIBLIOTECA</t>
+  </si>
+  <si>
+    <t>BILLARES</t>
+  </si>
+  <si>
+    <t>BODEGA</t>
+  </si>
+  <si>
+    <t>CABAÑA</t>
+  </si>
+  <si>
+    <t>CAMPO DE GOLF</t>
+  </si>
+  <si>
+    <t>CANTINA CABARET</t>
+  </si>
+  <si>
+    <t>CARCEL</t>
+  </si>
+  <si>
+    <t>CARNICERIA</t>
+  </si>
+  <si>
+    <t>CASA HABITACION</t>
+  </si>
+  <si>
+    <t>CASA HOGAR</t>
+  </si>
+  <si>
+    <t>CASETA DE POLICIA</t>
+  </si>
+  <si>
+    <t>CASETA DE VIGILANCIA</t>
+  </si>
+  <si>
+    <t>CENTRAL ELECTRICA</t>
+  </si>
+  <si>
+    <t>CLINICA</t>
+  </si>
+  <si>
+    <t>CLUB</t>
+  </si>
+  <si>
+    <t>COCHERA</t>
+  </si>
+  <si>
+    <t>COMERCIO</t>
+  </si>
+  <si>
+    <t>COMITE EJIDAL</t>
+  </si>
+  <si>
+    <t>CONSULTORIO MEDICO</t>
+  </si>
+  <si>
+    <t>CONVENTO</t>
+  </si>
+  <si>
+    <t>CUARTEL DE BOMBEROS</t>
+  </si>
+  <si>
+    <t>DEPOSITO DE AGUA</t>
+  </si>
+  <si>
+    <t>DIREC DE TRANSITO</t>
+  </si>
+  <si>
+    <t>DISPENSARIO</t>
+  </si>
+  <si>
+    <t>EMPACADORA</t>
+  </si>
+  <si>
+    <t>EN CONSTRUCCION</t>
+  </si>
+  <si>
+    <t>ERIAZO</t>
+  </si>
+  <si>
+    <t>ESCUELA PARTICULAR</t>
+  </si>
+  <si>
+    <t>ESCUELA PUBLICA</t>
+  </si>
+  <si>
+    <t>ESTABLO</t>
+  </si>
+  <si>
+    <t>ESTACION FFCC</t>
+  </si>
+  <si>
+    <t>ESTADIO</t>
+  </si>
+  <si>
+    <t>FABRICAS</t>
+  </si>
+  <si>
+    <t>FARMACIA</t>
+  </si>
+  <si>
+    <t>FRUTERIA</t>
+  </si>
+  <si>
+    <t>GALERA</t>
+  </si>
+  <si>
+    <t>GASERA</t>
+  </si>
+  <si>
+    <t>GASOLINERA</t>
+  </si>
+  <si>
+    <t>GUARDERIA</t>
+  </si>
+  <si>
+    <t>HOSPITAL</t>
+  </si>
+  <si>
+    <t>HOTEL</t>
+  </si>
+  <si>
+    <t>HUERTA</t>
+  </si>
+  <si>
+    <t>HUMEDAD</t>
+  </si>
+  <si>
+    <t>IGLESIAS</t>
+  </si>
+  <si>
+    <t>INSTALACIONES DEPORTIVAS</t>
+  </si>
+  <si>
+    <t>JARDIN</t>
+  </si>
+  <si>
+    <t>KIOSCO</t>
+  </si>
+  <si>
+    <t>LABORATORIO</t>
+  </si>
+  <si>
+    <t>LADRILLERA</t>
+  </si>
+  <si>
+    <t>LAVANDERIA PUBLICA</t>
+  </si>
+  <si>
+    <t>LICORERIA VINATERIA</t>
+  </si>
+  <si>
+    <t>LIENZO CHARRO</t>
+  </si>
+  <si>
+    <t>MADERERIA</t>
+  </si>
+  <si>
+    <t>MERCADO</t>
+  </si>
+  <si>
+    <t>MOLINO</t>
+  </si>
+  <si>
+    <t>MONTE ALTO</t>
+  </si>
+  <si>
+    <t>MONTE BAJO</t>
+  </si>
+  <si>
+    <t>MONUMENTO HISTORICO</t>
+  </si>
+  <si>
+    <t>NAVE INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>NO CLASIFICA</t>
+  </si>
+  <si>
+    <t>OFICINA DE VENTAS</t>
+  </si>
+  <si>
+    <t>OFICINAS</t>
+  </si>
+  <si>
+    <t>OFICINAS DE GOBIERNO</t>
+  </si>
+  <si>
+    <t>OFICINAS GENERALES</t>
+  </si>
+  <si>
+    <t>PANTEON</t>
+  </si>
+  <si>
+    <t>PELUQUERIA</t>
+  </si>
+  <si>
+    <t>PENSION AUTOMOVILES</t>
+  </si>
+  <si>
+    <t>PENTH HOUSE</t>
+  </si>
+  <si>
+    <t>PLANTA INDUSTRIAL</t>
+  </si>
+  <si>
+    <t>PLANTA TRATADORA DE AGUA</t>
+  </si>
+  <si>
+    <t>PLAZA CIVICA</t>
+  </si>
+  <si>
+    <t>PLAZA DE TOROS</t>
+  </si>
+  <si>
+    <t>POZO PROFUNDO</t>
+  </si>
+  <si>
+    <t>PRESIDENCIA MPAL</t>
+  </si>
+  <si>
+    <t>PROPIEDAD FEDERAL</t>
+  </si>
+  <si>
+    <t>RADIODIFUSORA</t>
+  </si>
+  <si>
+    <t>RASTRO</t>
+  </si>
+  <si>
+    <t>RESTAURANTE</t>
+  </si>
+  <si>
+    <t>RIEGO MECANICO</t>
+  </si>
+  <si>
+    <t>RIEGO POR GRAVEDAD</t>
+  </si>
+  <si>
+    <t>RUINAS</t>
+  </si>
+  <si>
+    <t>SALA DE BELLEZA</t>
+  </si>
+  <si>
+    <t>SALA DE ESPECTACULOS</t>
+  </si>
+  <si>
+    <t>SALON DE FIESTAS</t>
+  </si>
+  <si>
+    <t>SASTRERIA</t>
+  </si>
+  <si>
+    <t>SILVOPASTORIL</t>
+  </si>
+  <si>
+    <t>SIN USO DE PREDIO</t>
+  </si>
+  <si>
+    <t>SINDICATO</t>
+  </si>
+  <si>
+    <t>SUPERMERCADO</t>
+  </si>
+  <si>
+    <t>TALLER</t>
+  </si>
+  <si>
+    <t>TANQUE METALICO</t>
+  </si>
+  <si>
+    <t>TEMPORAL DE PRIMERA</t>
+  </si>
+  <si>
+    <t>TEMPORAL DE SEGUNDA</t>
+  </si>
+  <si>
+    <t>TEMPORAL DE TERCERA</t>
+  </si>
+  <si>
+    <t>TENERIA</t>
+  </si>
+  <si>
+    <t>TERMINAL DE CAMIONES</t>
+  </si>
+  <si>
+    <t>TINTORERIA</t>
+  </si>
+  <si>
+    <t>UNIDAD DEPORTIVA</t>
+  </si>
+  <si>
+    <t>UNIDAD HOGAR</t>
+  </si>
+  <si>
+    <t>USO COMERCIAL</t>
+  </si>
+  <si>
+    <t>VECINDAD</t>
+  </si>
+  <si>
+    <t>VETERINARIA</t>
+  </si>
+  <si>
+    <t>VIVERO</t>
+  </si>
+  <si>
+    <t>ZAHURDA</t>
+  </si>
+  <si>
+    <t>ZAPATERIA</t>
+  </si>
+  <si>
+    <t>ZOOLOGICO</t>
+  </si>
+  <si>
+    <t>INTERMEDIO</t>
+  </si>
+  <si>
+    <t>TRANSVERSAL CON FRENTES NO CONTIGUOS</t>
+  </si>
+  <si>
+    <t>CABECERA</t>
+  </si>
+  <si>
+    <t>MANZANERO</t>
+  </si>
+  <si>
+    <t>INTERIOR</t>
   </si>
 </sst>
 </file>
@@ -744,7 +1720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7806A9-AE76-44CF-993F-CC0D365B724C}">
-  <dimension ref="A1:CD3"/>
+  <dimension ref="A1:CD5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -761,7 +1737,7 @@
     <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.88671875" customWidth="1"/>
     <col min="21" max="21" width="20.21875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="15" bestFit="1" customWidth="1"/>
@@ -1153,6 +2129,14 @@
       <c r="BS3" s="7"/>
       <c r="BV3" s="7"/>
     </row>
+    <row r="4" spans="1:82" x14ac:dyDescent="0.3">
+      <c r="BS4" s="7"/>
+      <c r="BV4" s="7"/>
+    </row>
+    <row r="5" spans="1:82" x14ac:dyDescent="0.3">
+      <c r="BS5" s="7"/>
+      <c r="BV5" s="7"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="BW1:CC1"/>
@@ -1165,5 +2149,1628 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="28">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{37BD0220-9E51-45BA-A265-39BE25F7FCC8}">
+          <x14:formula1>
+            <xm:f>Hoja2!$A$2:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>P3:P1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E50DB94-E1AA-4CE4-ADEF-83A1F4AB5B43}">
+          <x14:formula1>
+            <xm:f>Hoja2!$AC$2:$AC$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>C3:C1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DDEB57E5-153F-4ED9-8C8C-C1FBBD8715F0}">
+          <x14:formula1>
+            <xm:f>Hoja2!$B$2:$B$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>Q3:Q1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E07B1B75-AF03-4A8D-BC24-5721557FF61A}">
+          <x14:formula1>
+            <xm:f>Hoja2!$C$2:$C$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>S3:S1048576 AP3:AP1048576 AQ3:AQ1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{41BB7C65-DC93-4292-81A0-F268D8A02A18}">
+          <x14:formula1>
+            <xm:f>Hoja2!$D$2:$D$45</xm:f>
+          </x14:formula1>
+          <xm:sqref>T3:T1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D9C52FE-6D55-407E-8C4B-88B2DEF94573}">
+          <x14:formula1>
+            <xm:f>Hoja2!$E$2:$E$31</xm:f>
+          </x14:formula1>
+          <xm:sqref>V3:V1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{84E5F63A-A4AB-47B5-97BA-AA3C8554A144}">
+          <x14:formula1>
+            <xm:f>Hoja2!$F$2:$F$26</xm:f>
+          </x14:formula1>
+          <xm:sqref>AN3:AN1048576 AO3:AO1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7D33DAEA-F9F3-4874-B861-42A021DC99B1}">
+          <x14:formula1>
+            <xm:f>Hoja2!$H$2:$H$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>AV3:AV1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{161264C7-A5E3-4F61-A614-028D62F3EC0E}">
+          <x14:formula1>
+            <xm:f>Hoja2!$I$2:$I$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>AW3:AW1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{795EBF0F-0DAD-4EB9-A428-BD50873910D0}">
+          <x14:formula1>
+            <xm:f>Hoja2!$J$2:$J$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>AX3:AX1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{28A1E571-1CEC-47BF-825E-67A9E930A0D3}">
+          <x14:formula1>
+            <xm:f>Hoja2!$K$2:$K$11</xm:f>
+          </x14:formula1>
+          <xm:sqref>AY3:AY1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F2DCA628-14C7-4F71-A7C2-378A86B56965}">
+          <x14:formula1>
+            <xm:f>Hoja2!$L$2:$L$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>AZ3:AZ1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25227AEB-E170-440B-A489-C54B8AAA71EE}">
+          <x14:formula1>
+            <xm:f>Hoja2!$M$2:$M$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>BA3:BA1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{14392394-449F-4C32-B560-7CCB1753B746}">
+          <x14:formula1>
+            <xm:f>Hoja2!$N$2:$N$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>BB3:BB1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7144E9CC-E537-4DC0-B364-139231DFAEF2}">
+          <x14:formula1>
+            <xm:f>Hoja2!$O$2:$O$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BC3:BC1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{22524E45-CF71-4F27-95AC-5851CBA321A6}">
+          <x14:formula1>
+            <xm:f>Hoja2!$P$2:$P$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>BD3:BD1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{46DF2204-513F-4B04-B29F-399B0D420994}">
+          <x14:formula1>
+            <xm:f>Hoja2!$Q$2:$Q$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>BE3:BE1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{66E24F7D-787B-4D0F-85D0-6816BB1C4822}">
+          <x14:formula1>
+            <xm:f>Hoja2!$R$2:$R$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BF3:BF1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5F22308-7CEA-4033-995C-256C6A7FAD4A}">
+          <x14:formula1>
+            <xm:f>Hoja2!$S$2:$S$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BG3:BG1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{048FD807-791D-4C41-9CAE-8C262B2803EA}">
+          <x14:formula1>
+            <xm:f>Hoja2!$T$2:$T$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>BH3:BH1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7CA12FC9-A5C1-479E-B2EE-19C704ABBAB2}">
+          <x14:formula1>
+            <xm:f>Hoja2!$U$2:$U$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>BI3:BI1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E3AB702-C42C-4122-9A12-001CB2150602}">
+          <x14:formula1>
+            <xm:f>Hoja2!$V$2:$V$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BJ3:BJ1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9BC56ED0-C878-4B70-AF59-878EF8AA865E}">
+          <x14:formula1>
+            <xm:f>Hoja2!$W$2:$W$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BK3:BK1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0E1A2C55-058E-4225-A3E9-B4F625D85399}">
+          <x14:formula1>
+            <xm:f>Hoja2!$X$2:$X$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>BL3:BL1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7BF7C810-BC07-467A-B909-741F16C106B4}">
+          <x14:formula1>
+            <xm:f>Hoja2!$Y$2:$Y$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>BM3:BM1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{60069B37-3CC2-4FE5-ABC6-4FCA59061E75}">
+          <x14:formula1>
+            <xm:f>Hoja2!$Z$2:$Z$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>BN3:BN1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4CA88649-FA21-4E18-8525-72E3D0112FE0}">
+          <x14:formula1>
+            <xm:f>Hoja2!$AA$2:$AA$126</xm:f>
+          </x14:formula1>
+          <xm:sqref>BS3:BS1048576 BT3:BT1048576 BU3:BU1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3172409-A8B4-45E9-A35A-A489AFE1480C}">
+          <x14:formula1>
+            <xm:f>Hoja2!$AB$2:$AB$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>BV3:BV1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F97A134-8EDF-4290-8B44-20FD0F25837A}">
+  <dimension ref="A1:AC126"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="4.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1" t="s">
+        <v>62</v>
+      </c>
+      <c r="O1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>65</v>
+      </c>
+      <c r="R1" t="s">
+        <v>66</v>
+      </c>
+      <c r="S1" t="s">
+        <v>67</v>
+      </c>
+      <c r="T1" t="s">
+        <v>68</v>
+      </c>
+      <c r="U1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V1" t="s">
+        <v>70</v>
+      </c>
+      <c r="W1" t="s">
+        <v>71</v>
+      </c>
+      <c r="X1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G2" t="s">
+        <v>202</v>
+      </c>
+      <c r="H2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" t="s">
+        <v>98</v>
+      </c>
+      <c r="M2" t="s">
+        <v>98</v>
+      </c>
+      <c r="N2" t="s">
+        <v>98</v>
+      </c>
+      <c r="O2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>98</v>
+      </c>
+      <c r="R2" t="s">
+        <v>98</v>
+      </c>
+      <c r="S2" t="s">
+        <v>98</v>
+      </c>
+      <c r="T2" t="s">
+        <v>98</v>
+      </c>
+      <c r="U2" t="s">
+        <v>98</v>
+      </c>
+      <c r="V2" t="s">
+        <v>98</v>
+      </c>
+      <c r="W2" t="s">
+        <v>98</v>
+      </c>
+      <c r="X2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>411</v>
+      </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G3" t="s">
+        <v>203</v>
+      </c>
+      <c r="H3" t="s">
+        <v>212</v>
+      </c>
+      <c r="I3" t="s">
+        <v>216</v>
+      </c>
+      <c r="J3" t="s">
+        <v>221</v>
+      </c>
+      <c r="K3" t="s">
+        <v>227</v>
+      </c>
+      <c r="L3" t="s">
+        <v>236</v>
+      </c>
+      <c r="M3" t="s">
+        <v>242</v>
+      </c>
+      <c r="N3" t="s">
+        <v>247</v>
+      </c>
+      <c r="O3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P3" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>261</v>
+      </c>
+      <c r="R3" t="s">
+        <v>265</v>
+      </c>
+      <c r="S3" t="s">
+        <v>268</v>
+      </c>
+      <c r="T3" t="s">
+        <v>271</v>
+      </c>
+      <c r="U3" t="s">
+        <v>275</v>
+      </c>
+      <c r="V3" t="s">
+        <v>278</v>
+      </c>
+      <c r="W3" t="s">
+        <v>281</v>
+      </c>
+      <c r="X3" t="s">
+        <v>284</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>278</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>287</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>290</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AC3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G4" t="s">
+        <v>204</v>
+      </c>
+      <c r="H4" t="s">
+        <v>213</v>
+      </c>
+      <c r="I4" t="s">
+        <v>217</v>
+      </c>
+      <c r="J4" t="s">
+        <v>222</v>
+      </c>
+      <c r="K4" t="s">
+        <v>228</v>
+      </c>
+      <c r="L4" t="s">
+        <v>237</v>
+      </c>
+      <c r="M4" t="s">
+        <v>243</v>
+      </c>
+      <c r="N4" t="s">
+        <v>248</v>
+      </c>
+      <c r="O4" t="s">
+        <v>254</v>
+      </c>
+      <c r="P4" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>262</v>
+      </c>
+      <c r="R4" t="s">
+        <v>266</v>
+      </c>
+      <c r="S4" t="s">
+        <v>269</v>
+      </c>
+      <c r="T4" t="s">
+        <v>272</v>
+      </c>
+      <c r="U4" t="s">
+        <v>276</v>
+      </c>
+      <c r="V4" t="s">
+        <v>279</v>
+      </c>
+      <c r="W4" t="s">
+        <v>282</v>
+      </c>
+      <c r="X4" t="s">
+        <v>285</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>286</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>288</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>291</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F5" t="s">
+        <v>181</v>
+      </c>
+      <c r="G5" t="s">
+        <v>205</v>
+      </c>
+      <c r="H5" t="s">
+        <v>214</v>
+      </c>
+      <c r="I5" t="s">
+        <v>218</v>
+      </c>
+      <c r="J5" t="s">
+        <v>223</v>
+      </c>
+      <c r="K5" t="s">
+        <v>229</v>
+      </c>
+      <c r="L5" t="s">
+        <v>238</v>
+      </c>
+      <c r="M5" t="s">
+        <v>244</v>
+      </c>
+      <c r="N5" t="s">
+        <v>249</v>
+      </c>
+      <c r="O5" t="s">
+        <v>255</v>
+      </c>
+      <c r="P5" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>263</v>
+      </c>
+      <c r="R5" t="s">
+        <v>267</v>
+      </c>
+      <c r="S5" t="s">
+        <v>270</v>
+      </c>
+      <c r="T5" t="s">
+        <v>243</v>
+      </c>
+      <c r="U5" t="s">
+        <v>228</v>
+      </c>
+      <c r="V5" t="s">
+        <v>280</v>
+      </c>
+      <c r="W5" t="s">
+        <v>283</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>289</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>292</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" t="s">
+        <v>182</v>
+      </c>
+      <c r="G6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" t="s">
+        <v>215</v>
+      </c>
+      <c r="I6" t="s">
+        <v>219</v>
+      </c>
+      <c r="J6" t="s">
+        <v>224</v>
+      </c>
+      <c r="K6" t="s">
+        <v>230</v>
+      </c>
+      <c r="L6" t="s">
+        <v>239</v>
+      </c>
+      <c r="M6" t="s">
+        <v>245</v>
+      </c>
+      <c r="N6" t="s">
+        <v>250</v>
+      </c>
+      <c r="P6" t="s">
+        <v>255</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>264</v>
+      </c>
+      <c r="T6" t="s">
+        <v>273</v>
+      </c>
+      <c r="U6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>293</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G7" t="s">
+        <v>206</v>
+      </c>
+      <c r="I7" t="s">
+        <v>220</v>
+      </c>
+      <c r="J7" t="s">
+        <v>225</v>
+      </c>
+      <c r="K7" t="s">
+        <v>231</v>
+      </c>
+      <c r="L7" t="s">
+        <v>240</v>
+      </c>
+      <c r="M7" t="s">
+        <v>246</v>
+      </c>
+      <c r="N7" t="s">
+        <v>251</v>
+      </c>
+      <c r="P7" t="s">
+        <v>258</v>
+      </c>
+      <c r="T7" t="s">
+        <v>274</v>
+      </c>
+      <c r="U7" t="s">
+        <v>254</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>294</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G8" t="s">
+        <v>207</v>
+      </c>
+      <c r="I8" t="s">
+        <v>220</v>
+      </c>
+      <c r="J8" t="s">
+        <v>226</v>
+      </c>
+      <c r="K8" t="s">
+        <v>232</v>
+      </c>
+      <c r="L8" t="s">
+        <v>241</v>
+      </c>
+      <c r="N8" t="s">
+        <v>252</v>
+      </c>
+      <c r="P8" t="s">
+        <v>259</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" t="s">
+        <v>185</v>
+      </c>
+      <c r="G9" t="s">
+        <v>208</v>
+      </c>
+      <c r="K9" t="s">
+        <v>233</v>
+      </c>
+      <c r="P9" t="s">
+        <v>260</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" t="s">
+        <v>160</v>
+      </c>
+      <c r="F10" t="s">
+        <v>186</v>
+      </c>
+      <c r="G10" t="s">
+        <v>209</v>
+      </c>
+      <c r="K10" t="s">
+        <v>234</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F11" t="s">
+        <v>187</v>
+      </c>
+      <c r="G11" t="s">
+        <v>210</v>
+      </c>
+      <c r="K11" t="s">
+        <v>235</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F12" t="s">
+        <v>188</v>
+      </c>
+      <c r="G12" t="s">
+        <v>211</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" t="s">
+        <v>163</v>
+      </c>
+      <c r="F13" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>121</v>
+      </c>
+      <c r="E14" t="s">
+        <v>164</v>
+      </c>
+      <c r="F14" t="s">
+        <v>189</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" t="s">
+        <v>190</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F16" t="s">
+        <v>191</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="17" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" t="s">
+        <v>166</v>
+      </c>
+      <c r="F17" t="s">
+        <v>192</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="18" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" t="s">
+        <v>167</v>
+      </c>
+      <c r="F18" t="s">
+        <v>193</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="19" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D19" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" t="s">
+        <v>120</v>
+      </c>
+      <c r="F19" t="s">
+        <v>194</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="20" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>127</v>
+      </c>
+      <c r="E20" t="s">
+        <v>168</v>
+      </c>
+      <c r="F20" t="s">
+        <v>195</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="21" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>128</v>
+      </c>
+      <c r="E21" t="s">
+        <v>169</v>
+      </c>
+      <c r="F21" t="s">
+        <v>196</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="22" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
+        <v>129</v>
+      </c>
+      <c r="E22" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" t="s">
+        <v>197</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="23" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D23" t="s">
+        <v>130</v>
+      </c>
+      <c r="E23" t="s">
+        <v>171</v>
+      </c>
+      <c r="F23" t="s">
+        <v>198</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="24" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D24" t="s">
+        <v>131</v>
+      </c>
+      <c r="E24" t="s">
+        <v>172</v>
+      </c>
+      <c r="F24" t="s">
+        <v>199</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="25" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D25" t="s">
+        <v>132</v>
+      </c>
+      <c r="E25" t="s">
+        <v>173</v>
+      </c>
+      <c r="F25" t="s">
+        <v>200</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="26" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D26" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" t="s">
+        <v>174</v>
+      </c>
+      <c r="F26" t="s">
+        <v>201</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="27" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D27" t="s">
+        <v>134</v>
+      </c>
+      <c r="E27" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="28" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>135</v>
+      </c>
+      <c r="E28" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="29" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
+        <v>136</v>
+      </c>
+      <c r="E29" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="30" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D30" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" t="s">
+        <v>176</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="31" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D31" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="32" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D32" t="s">
+        <v>139</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="33" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D33" t="s">
+        <v>140</v>
+      </c>
+      <c r="AA33" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="34" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D34" t="s">
+        <v>141</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="35" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D35" t="s">
+        <v>142</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="36" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D36" t="s">
+        <v>143</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="37" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D37" t="s">
+        <v>144</v>
+      </c>
+      <c r="AA37" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="38" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D38" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA38" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="39" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D39" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA39" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="40" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D40" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA40" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="41" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D41" t="s">
+        <v>148</v>
+      </c>
+      <c r="AA41" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="42" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D42" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA42" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="43" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D43" t="s">
+        <v>150</v>
+      </c>
+      <c r="AA43" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="44" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D44" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA44" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="45" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="D45" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA45" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="46" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="AA46" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="47" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="AA47" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="48" spans="4:27" x14ac:dyDescent="0.3">
+      <c r="AA48" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="49" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA49" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="50" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA50" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="51" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA51" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="52" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA52" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="53" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA53" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="54" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA54" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="55" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA55" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="56" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA56" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="57" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA57" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="58" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA58" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="59" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA59" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="60" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA60" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="61" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA61" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="62" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA62" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="63" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA63" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA64" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="65" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA65" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="66" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA66" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="67" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA67" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="68" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA68" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="69" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA69" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="70" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA70" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="71" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA71" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="72" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA72" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="73" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA73" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="74" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA74" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="75" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA75" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="76" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA76" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="77" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA77" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="78" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA78" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="79" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA79" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="80" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA80" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="81" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA81" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="82" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA82" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="83" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA83" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="84" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA84" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="85" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA85" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="86" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA86" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="87" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA87" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="88" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA88" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="89" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA89" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="90" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA90" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="91" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA91" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="92" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA92" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="93" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA93" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="94" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA94" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="95" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA95" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="96" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA96" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="97" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA97" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="98" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA98" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA99" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="100" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA100" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="101" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA101" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="102" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA102" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="103" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA103" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="104" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA104" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="105" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA105" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="106" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA106" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="107" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA107" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="108" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA108" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="109" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA109" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="110" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA110" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="111" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA111" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="112" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA112" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="113" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA113" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="114" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA114" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="115" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA115" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="116" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA116" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="117" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA117" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="118" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA118" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="119" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA119" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="120" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA120" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="121" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA121" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="122" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA122" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="123" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA123" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="124" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA124" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="125" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA125" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="126" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA126" t="s">
+        <v>410</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se finaliza área de descripción del predio, se agregan sectores a oficinas, correcciónes generales en valuacion
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sgc\storage\app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A72C4D4-1D41-4E94-901C-118B8DBF81F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C55AB68-2AA9-4968-B717-76DAA72B4AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{28BFEBC5-EF34-42C7-846D-BB644F26337B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="417">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -1283,6 +1283,9 @@
   </si>
   <si>
     <t>INTERIOR</t>
+  </si>
+  <si>
+    <t>predio</t>
   </si>
 </sst>
 </file>
@@ -1720,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7806A9-AE76-44CF-993F-CC0D365B724C}">
-  <dimension ref="A1:CD5"/>
+  <dimension ref="A1:CE5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -1733,49 +1736,50 @@
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.88671875" customWidth="1"/>
-    <col min="21" max="21" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.88671875" style="7" customWidth="1"/>
-    <col min="40" max="40" width="16" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="26" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="49" max="50" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="11.5546875" style="7"/>
-    <col min="68" max="68" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="20.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="16" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="31" customWidth="1"/>
+    <col min="11" max="11" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.88671875" customWidth="1"/>
+    <col min="22" max="22" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20.88671875" style="7" customWidth="1"/>
+    <col min="41" max="41" width="16" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="26" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="50" max="51" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="11.5546875" style="7"/>
+    <col min="69" max="69" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="20.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:82" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:83" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1792,19 +1796,19 @@
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
       <c r="L1" s="8"/>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="8"/>
+      <c r="N1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="10"/>
       <c r="O1" s="10"/>
       <c r="P1" s="10"/>
       <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
-      <c r="T1" s="11" t="s">
+      <c r="T1" s="10"/>
+      <c r="U1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="U1" s="11"/>
       <c r="V1" s="11"/>
       <c r="W1" s="11"/>
       <c r="X1" s="11"/>
@@ -1822,13 +1826,13 @@
       <c r="AJ1" s="11"/>
       <c r="AK1" s="11"/>
       <c r="AL1" s="11"/>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="11"/>
+      <c r="AN1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AN1" s="12" t="s">
+      <c r="AO1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="AO1" s="12"/>
       <c r="AP1" s="12"/>
       <c r="AQ1" s="12"/>
       <c r="AR1" s="12"/>
@@ -1854,30 +1858,31 @@
       <c r="BL1" s="12"/>
       <c r="BM1" s="12"/>
       <c r="BN1" s="12"/>
-      <c r="BO1" s="10" t="s">
+      <c r="BO1" s="12"/>
+      <c r="BP1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="BP1" s="10"/>
       <c r="BQ1" s="10"/>
       <c r="BR1" s="10"/>
       <c r="BS1" s="10"/>
       <c r="BT1" s="10"/>
       <c r="BU1" s="10"/>
       <c r="BV1" s="10"/>
-      <c r="BW1" s="8" t="s">
+      <c r="BW1" s="10"/>
+      <c r="BX1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="BX1" s="8"/>
       <c r="BY1" s="8"/>
       <c r="BZ1" s="8"/>
       <c r="CA1" s="8"/>
       <c r="CB1" s="8"/>
       <c r="CC1" s="8"/>
-      <c r="CD1" s="2" t="s">
+      <c r="CD1" s="8"/>
+      <c r="CE1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:82" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:83" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -1909,243 +1914,246 @@
         <v>18</v>
       </c>
       <c r="K2" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AM2" s="5" t="s">
+      <c r="AN2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AW2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="BO2" s="5" t="s">
+      <c r="BP2" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="BP2" s="5" t="s">
+      <c r="BQ2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="BQ2" s="5" t="s">
+      <c r="BR2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="BR2" s="5" t="s">
+      <c r="BS2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="BS2" s="4" t="s">
+      <c r="BT2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="BT2" s="4" t="s">
+      <c r="BU2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="BU2" s="4" t="s">
+      <c r="BV2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="BV2" s="4" t="s">
+      <c r="BW2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="BW2" s="4" t="s">
+      <c r="BX2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="BX2" s="4" t="s">
+      <c r="BY2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="BY2" s="4" t="s">
+      <c r="BZ2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="BZ2" s="4" t="s">
+      <c r="CA2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="CA2" s="4" t="s">
+      <c r="CB2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="CB2" s="4" t="s">
+      <c r="CC2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="CC2" s="4" t="s">
+      <c r="CD2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="CD2" s="4" t="s">
+      <c r="CE2" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:82" x14ac:dyDescent="0.3">
-      <c r="BS3" s="7"/>
-      <c r="BV3" s="7"/>
-    </row>
-    <row r="4" spans="1:82" x14ac:dyDescent="0.3">
-      <c r="BS4" s="7"/>
-      <c r="BV4" s="7"/>
-    </row>
-    <row r="5" spans="1:82" x14ac:dyDescent="0.3">
-      <c r="BS5" s="7"/>
-      <c r="BV5" s="7"/>
+    <row r="3" spans="1:83" x14ac:dyDescent="0.3">
+      <c r="BT3" s="7"/>
+      <c r="BW3" s="7"/>
+    </row>
+    <row r="4" spans="1:83" x14ac:dyDescent="0.3">
+      <c r="BT4" s="7"/>
+      <c r="BW4" s="7"/>
+    </row>
+    <row r="5" spans="1:83" x14ac:dyDescent="0.3">
+      <c r="BT5" s="7"/>
+      <c r="BW5" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="BW1:CC1"/>
+    <mergeCell ref="BX1:CD1"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:L1"/>
-    <mergeCell ref="M1:S1"/>
-    <mergeCell ref="T1:AL1"/>
-    <mergeCell ref="AN1:BN1"/>
-    <mergeCell ref="BO1:BV1"/>
+    <mergeCell ref="E1:M1"/>
+    <mergeCell ref="N1:T1"/>
+    <mergeCell ref="U1:AM1"/>
+    <mergeCell ref="AO1:BO1"/>
+    <mergeCell ref="BP1:BW1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2156,7 +2164,7 @@
           <x14:formula1>
             <xm:f>Hoja2!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>P3:P1048576</xm:sqref>
+          <xm:sqref>Q3:Q1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E50DB94-E1AA-4CE4-ADEF-83A1F4AB5B43}">
           <x14:formula1>
@@ -2168,157 +2176,157 @@
           <x14:formula1>
             <xm:f>Hoja2!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>Q3:Q1048576</xm:sqref>
+          <xm:sqref>R3:R1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E07B1B75-AF03-4A8D-BC24-5721557FF61A}">
           <x14:formula1>
             <xm:f>Hoja2!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>S3:S1048576 AP3:AP1048576 AQ3:AQ1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576</xm:sqref>
+          <xm:sqref>T3:T1048576 AQ3:AQ1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576 AV3:AV1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{41BB7C65-DC93-4292-81A0-F268D8A02A18}">
           <x14:formula1>
             <xm:f>Hoja2!$D$2:$D$45</xm:f>
           </x14:formula1>
-          <xm:sqref>T3:T1048576</xm:sqref>
+          <xm:sqref>U3:U1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D9C52FE-6D55-407E-8C4B-88B2DEF94573}">
           <x14:formula1>
             <xm:f>Hoja2!$E$2:$E$31</xm:f>
           </x14:formula1>
-          <xm:sqref>V3:V1048576</xm:sqref>
+          <xm:sqref>W3:W1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{84E5F63A-A4AB-47B5-97BA-AA3C8554A144}">
           <x14:formula1>
             <xm:f>Hoja2!$F$2:$F$26</xm:f>
           </x14:formula1>
-          <xm:sqref>AN3:AN1048576 AO3:AO1048576</xm:sqref>
+          <xm:sqref>AO3:AO1048576 AP3:AP1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7D33DAEA-F9F3-4874-B861-42A021DC99B1}">
           <x14:formula1>
             <xm:f>Hoja2!$H$2:$H$6</xm:f>
           </x14:formula1>
-          <xm:sqref>AV3:AV1048576</xm:sqref>
+          <xm:sqref>AW3:AW1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{161264C7-A5E3-4F61-A614-028D62F3EC0E}">
           <x14:formula1>
             <xm:f>Hoja2!$I$2:$I$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AW3:AW1048576</xm:sqref>
+          <xm:sqref>AX3:AX1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{795EBF0F-0DAD-4EB9-A428-BD50873910D0}">
           <x14:formula1>
             <xm:f>Hoja2!$J$2:$J$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AX3:AX1048576</xm:sqref>
+          <xm:sqref>AY3:AY1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{28A1E571-1CEC-47BF-825E-67A9E930A0D3}">
           <x14:formula1>
             <xm:f>Hoja2!$K$2:$K$11</xm:f>
           </x14:formula1>
-          <xm:sqref>AY3:AY1048576</xm:sqref>
+          <xm:sqref>AZ3:AZ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F2DCA628-14C7-4F71-A7C2-378A86B56965}">
           <x14:formula1>
             <xm:f>Hoja2!$L$2:$L$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AZ3:AZ1048576</xm:sqref>
+          <xm:sqref>BA3:BA1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25227AEB-E170-440B-A489-C54B8AAA71EE}">
           <x14:formula1>
             <xm:f>Hoja2!$M$2:$M$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BA3:BA1048576</xm:sqref>
+          <xm:sqref>BB3:BB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{14392394-449F-4C32-B560-7CCB1753B746}">
           <x14:formula1>
             <xm:f>Hoja2!$N$2:$N$8</xm:f>
           </x14:formula1>
-          <xm:sqref>BB3:BB1048576</xm:sqref>
+          <xm:sqref>BC3:BC1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7144E9CC-E537-4DC0-B364-139231DFAEF2}">
           <x14:formula1>
             <xm:f>Hoja2!$O$2:$O$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BC3:BC1048576</xm:sqref>
+          <xm:sqref>BD3:BD1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{22524E45-CF71-4F27-95AC-5851CBA321A6}">
           <x14:formula1>
             <xm:f>Hoja2!$P$2:$P$9</xm:f>
           </x14:formula1>
-          <xm:sqref>BD3:BD1048576</xm:sqref>
+          <xm:sqref>BE3:BE1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{46DF2204-513F-4B04-B29F-399B0D420994}">
           <x14:formula1>
             <xm:f>Hoja2!$Q$2:$Q$6</xm:f>
           </x14:formula1>
-          <xm:sqref>BE3:BE1048576</xm:sqref>
+          <xm:sqref>BF3:BF1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{66E24F7D-787B-4D0F-85D0-6816BB1C4822}">
           <x14:formula1>
             <xm:f>Hoja2!$R$2:$R$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BF3:BF1048576</xm:sqref>
+          <xm:sqref>BG3:BG1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5F22308-7CEA-4033-995C-256C6A7FAD4A}">
           <x14:formula1>
             <xm:f>Hoja2!$S$2:$S$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BG3:BG1048576</xm:sqref>
+          <xm:sqref>BH3:BH1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{048FD807-791D-4C41-9CAE-8C262B2803EA}">
           <x14:formula1>
             <xm:f>Hoja2!$T$2:$T$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BH3:BH1048576</xm:sqref>
+          <xm:sqref>BI3:BI1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7CA12FC9-A5C1-479E-B2EE-19C704ABBAB2}">
           <x14:formula1>
             <xm:f>Hoja2!$U$2:$U$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BI3:BI1048576</xm:sqref>
+          <xm:sqref>BJ3:BJ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E3AB702-C42C-4122-9A12-001CB2150602}">
           <x14:formula1>
             <xm:f>Hoja2!$V$2:$V$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BJ3:BJ1048576</xm:sqref>
+          <xm:sqref>BK3:BK1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9BC56ED0-C878-4B70-AF59-878EF8AA865E}">
           <x14:formula1>
             <xm:f>Hoja2!$W$2:$W$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BK3:BK1048576</xm:sqref>
+          <xm:sqref>BL3:BL1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0E1A2C55-058E-4225-A3E9-B4F625D85399}">
           <x14:formula1>
             <xm:f>Hoja2!$X$2:$X$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BL3:BL1048576</xm:sqref>
+          <xm:sqref>BM3:BM1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7BF7C810-BC07-467A-B909-741F16C106B4}">
           <x14:formula1>
             <xm:f>Hoja2!$Y$2:$Y$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BM3:BM1048576</xm:sqref>
+          <xm:sqref>BN3:BN1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{60069B37-3CC2-4FE5-ABC6-4FCA59061E75}">
           <x14:formula1>
             <xm:f>Hoja2!$Z$2:$Z$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BN3:BN1048576</xm:sqref>
+          <xm:sqref>BO3:BO1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4CA88649-FA21-4E18-8525-72E3D0112FE0}">
           <x14:formula1>
             <xm:f>Hoja2!$AA$2:$AA$126</xm:f>
           </x14:formula1>
-          <xm:sqref>BS3:BS1048576 BT3:BT1048576 BU3:BU1048576</xm:sqref>
+          <xm:sqref>BT3:BT1048576 BU3:BU1048576 BV3:BV1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3172409-A8B4-45E9-A35A-A489AFE1480C}">
           <x14:formula1>
             <xm:f>Hoja2!$AB$2:$AB$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BV3:BV1048576</xm:sqref>
+          <xm:sqref>BW3:BW1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se refactorizo tablas de avluos y predios, se removieron movimientos, se agregaron movimientos en tags de Auduiting
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sgc\storage\app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C55AB68-2AA9-4968-B717-76DAA72B4AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6368C403-09A6-4BA5-B04A-86DAE7E78030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{28BFEBC5-EF34-42C7-846D-BB644F26337B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="417">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -1723,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7806A9-AE76-44CF-993F-CC0D365B724C}">
-  <dimension ref="A1:CE5"/>
+  <dimension ref="A1:CF5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -1734,52 +1734,53 @@
     <col min="6" max="6" width="6.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.88671875" customWidth="1"/>
-    <col min="22" max="22" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="20.88671875" style="7" customWidth="1"/>
-    <col min="41" max="41" width="16" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="26" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="51" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="11.5546875" style="7"/>
-    <col min="69" max="69" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="20.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="16" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="31" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.88671875" customWidth="1"/>
+    <col min="23" max="23" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="20.88671875" style="7" customWidth="1"/>
+    <col min="42" max="42" width="16" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="26" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="51" max="52" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.5546875" style="7"/>
+    <col min="70" max="70" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="20.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="16" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:83" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:84" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1797,19 +1798,19 @@
       <c r="K1" s="8"/>
       <c r="L1" s="8"/>
       <c r="M1" s="8"/>
-      <c r="N1" s="10" t="s">
+      <c r="N1" s="8"/>
+      <c r="O1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="10"/>
       <c r="P1" s="10"/>
       <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10"/>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="10"/>
+      <c r="V1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="11"/>
       <c r="W1" s="11"/>
       <c r="X1" s="11"/>
       <c r="Y1" s="11"/>
@@ -1827,13 +1828,13 @@
       <c r="AK1" s="11"/>
       <c r="AL1" s="11"/>
       <c r="AM1" s="11"/>
-      <c r="AN1" s="1" t="s">
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AO1" s="12" t="s">
+      <c r="AP1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="AP1" s="12"/>
       <c r="AQ1" s="12"/>
       <c r="AR1" s="12"/>
       <c r="AS1" s="12"/>
@@ -1859,30 +1860,31 @@
       <c r="BM1" s="12"/>
       <c r="BN1" s="12"/>
       <c r="BO1" s="12"/>
-      <c r="BP1" s="10" t="s">
+      <c r="BP1" s="12"/>
+      <c r="BQ1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="BQ1" s="10"/>
       <c r="BR1" s="10"/>
       <c r="BS1" s="10"/>
       <c r="BT1" s="10"/>
       <c r="BU1" s="10"/>
       <c r="BV1" s="10"/>
       <c r="BW1" s="10"/>
-      <c r="BX1" s="8" t="s">
+      <c r="BX1" s="10"/>
+      <c r="BY1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="BY1" s="8"/>
       <c r="BZ1" s="8"/>
       <c r="CA1" s="8"/>
       <c r="CB1" s="8"/>
       <c r="CC1" s="8"/>
       <c r="CD1" s="8"/>
-      <c r="CE1" s="2" t="s">
+      <c r="CE1" s="8"/>
+      <c r="CF1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:83" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:84" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -1908,252 +1910,255 @@
         <v>16</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AN2" s="5" t="s">
+      <c r="AO2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="AW2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="BO2" s="4" t="s">
+      <c r="BP2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="BP2" s="5" t="s">
+      <c r="BQ2" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="BQ2" s="5" t="s">
+      <c r="BR2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="BR2" s="5" t="s">
+      <c r="BS2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="BS2" s="5" t="s">
+      <c r="BT2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="BT2" s="4" t="s">
+      <c r="BU2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="BU2" s="4" t="s">
+      <c r="BV2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="BV2" s="4" t="s">
+      <c r="BW2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="BW2" s="4" t="s">
+      <c r="BX2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="BX2" s="4" t="s">
+      <c r="BY2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="BY2" s="4" t="s">
+      <c r="BZ2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="BZ2" s="4" t="s">
+      <c r="CA2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="CA2" s="4" t="s">
+      <c r="CB2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="CB2" s="4" t="s">
+      <c r="CC2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="CC2" s="4" t="s">
+      <c r="CD2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="CD2" s="4" t="s">
+      <c r="CE2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="CE2" s="4" t="s">
+      <c r="CF2" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:83" x14ac:dyDescent="0.3">
-      <c r="BT3" s="7"/>
-      <c r="BW3" s="7"/>
-    </row>
-    <row r="4" spans="1:83" x14ac:dyDescent="0.3">
-      <c r="BT4" s="7"/>
-      <c r="BW4" s="7"/>
-    </row>
-    <row r="5" spans="1:83" x14ac:dyDescent="0.3">
-      <c r="BT5" s="7"/>
-      <c r="BW5" s="7"/>
+    <row r="3" spans="1:84" x14ac:dyDescent="0.3">
+      <c r="BU3" s="7"/>
+      <c r="BX3" s="7"/>
+    </row>
+    <row r="4" spans="1:84" x14ac:dyDescent="0.3">
+      <c r="BU4" s="7"/>
+      <c r="BX4" s="7"/>
+    </row>
+    <row r="5" spans="1:84" x14ac:dyDescent="0.3">
+      <c r="BU5" s="7"/>
+      <c r="BX5" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="BX1:CD1"/>
+    <mergeCell ref="BY1:CE1"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:M1"/>
-    <mergeCell ref="N1:T1"/>
-    <mergeCell ref="U1:AM1"/>
-    <mergeCell ref="AO1:BO1"/>
-    <mergeCell ref="BP1:BW1"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="O1:U1"/>
+    <mergeCell ref="V1:AN1"/>
+    <mergeCell ref="AP1:BP1"/>
+    <mergeCell ref="BQ1:BX1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2164,7 +2169,7 @@
           <x14:formula1>
             <xm:f>Hoja2!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>Q3:Q1048576</xm:sqref>
+          <xm:sqref>R3:R1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E50DB94-E1AA-4CE4-ADEF-83A1F4AB5B43}">
           <x14:formula1>
@@ -2176,157 +2181,157 @@
           <x14:formula1>
             <xm:f>Hoja2!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>R3:R1048576</xm:sqref>
+          <xm:sqref>S3:S1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E07B1B75-AF03-4A8D-BC24-5721557FF61A}">
           <x14:formula1>
             <xm:f>Hoja2!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>T3:T1048576 AQ3:AQ1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576 AV3:AV1048576</xm:sqref>
+          <xm:sqref>U3:U1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576 AV3:AV1048576 AW3:AW1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{41BB7C65-DC93-4292-81A0-F268D8A02A18}">
           <x14:formula1>
             <xm:f>Hoja2!$D$2:$D$45</xm:f>
           </x14:formula1>
-          <xm:sqref>U3:U1048576</xm:sqref>
+          <xm:sqref>V3:V1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D9C52FE-6D55-407E-8C4B-88B2DEF94573}">
           <x14:formula1>
             <xm:f>Hoja2!$E$2:$E$31</xm:f>
           </x14:formula1>
-          <xm:sqref>W3:W1048576</xm:sqref>
+          <xm:sqref>X3:X1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{84E5F63A-A4AB-47B5-97BA-AA3C8554A144}">
           <x14:formula1>
             <xm:f>Hoja2!$F$2:$F$26</xm:f>
           </x14:formula1>
-          <xm:sqref>AO3:AO1048576 AP3:AP1048576</xm:sqref>
+          <xm:sqref>AP3:AP1048576 AQ3:AQ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7D33DAEA-F9F3-4874-B861-42A021DC99B1}">
           <x14:formula1>
             <xm:f>Hoja2!$H$2:$H$6</xm:f>
           </x14:formula1>
-          <xm:sqref>AW3:AW1048576</xm:sqref>
+          <xm:sqref>AX3:AX1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{161264C7-A5E3-4F61-A614-028D62F3EC0E}">
           <x14:formula1>
             <xm:f>Hoja2!$I$2:$I$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AX3:AX1048576</xm:sqref>
+          <xm:sqref>AY3:AY1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{795EBF0F-0DAD-4EB9-A428-BD50873910D0}">
           <x14:formula1>
             <xm:f>Hoja2!$J$2:$J$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AY3:AY1048576</xm:sqref>
+          <xm:sqref>AZ3:AZ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{28A1E571-1CEC-47BF-825E-67A9E930A0D3}">
           <x14:formula1>
             <xm:f>Hoja2!$K$2:$K$11</xm:f>
           </x14:formula1>
-          <xm:sqref>AZ3:AZ1048576</xm:sqref>
+          <xm:sqref>BA3:BA1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F2DCA628-14C7-4F71-A7C2-378A86B56965}">
           <x14:formula1>
             <xm:f>Hoja2!$L$2:$L$8</xm:f>
           </x14:formula1>
-          <xm:sqref>BA3:BA1048576</xm:sqref>
+          <xm:sqref>BB3:BB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25227AEB-E170-440B-A489-C54B8AAA71EE}">
           <x14:formula1>
             <xm:f>Hoja2!$M$2:$M$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BB3:BB1048576</xm:sqref>
+          <xm:sqref>BC3:BC1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{14392394-449F-4C32-B560-7CCB1753B746}">
           <x14:formula1>
             <xm:f>Hoja2!$N$2:$N$8</xm:f>
           </x14:formula1>
-          <xm:sqref>BC3:BC1048576</xm:sqref>
+          <xm:sqref>BD3:BD1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7144E9CC-E537-4DC0-B364-139231DFAEF2}">
           <x14:formula1>
             <xm:f>Hoja2!$O$2:$O$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BD3:BD1048576</xm:sqref>
+          <xm:sqref>BE3:BE1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{22524E45-CF71-4F27-95AC-5851CBA321A6}">
           <x14:formula1>
             <xm:f>Hoja2!$P$2:$P$9</xm:f>
           </x14:formula1>
-          <xm:sqref>BE3:BE1048576</xm:sqref>
+          <xm:sqref>BF3:BF1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{46DF2204-513F-4B04-B29F-399B0D420994}">
           <x14:formula1>
             <xm:f>Hoja2!$Q$2:$Q$6</xm:f>
           </x14:formula1>
-          <xm:sqref>BF3:BF1048576</xm:sqref>
+          <xm:sqref>BG3:BG1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{66E24F7D-787B-4D0F-85D0-6816BB1C4822}">
           <x14:formula1>
             <xm:f>Hoja2!$R$2:$R$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BG3:BG1048576</xm:sqref>
+          <xm:sqref>BH3:BH1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5F22308-7CEA-4033-995C-256C6A7FAD4A}">
           <x14:formula1>
             <xm:f>Hoja2!$S$2:$S$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BH3:BH1048576</xm:sqref>
+          <xm:sqref>BI3:BI1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{048FD807-791D-4C41-9CAE-8C262B2803EA}">
           <x14:formula1>
             <xm:f>Hoja2!$T$2:$T$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BI3:BI1048576</xm:sqref>
+          <xm:sqref>BJ3:BJ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7CA12FC9-A5C1-479E-B2EE-19C704ABBAB2}">
           <x14:formula1>
             <xm:f>Hoja2!$U$2:$U$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BJ3:BJ1048576</xm:sqref>
+          <xm:sqref>BK3:BK1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E3AB702-C42C-4122-9A12-001CB2150602}">
           <x14:formula1>
             <xm:f>Hoja2!$V$2:$V$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BK3:BK1048576</xm:sqref>
+          <xm:sqref>BL3:BL1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9BC56ED0-C878-4B70-AF59-878EF8AA865E}">
           <x14:formula1>
             <xm:f>Hoja2!$W$2:$W$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BL3:BL1048576</xm:sqref>
+          <xm:sqref>BM3:BM1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0E1A2C55-058E-4225-A3E9-B4F625D85399}">
           <x14:formula1>
             <xm:f>Hoja2!$X$2:$X$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BM3:BM1048576</xm:sqref>
+          <xm:sqref>BN3:BN1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7BF7C810-BC07-467A-B909-741F16C106B4}">
           <x14:formula1>
             <xm:f>Hoja2!$Y$2:$Y$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BN3:BN1048576</xm:sqref>
+          <xm:sqref>BO3:BO1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{60069B37-3CC2-4FE5-ABC6-4FCA59061E75}">
           <x14:formula1>
             <xm:f>Hoja2!$Z$2:$Z$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BO3:BO1048576</xm:sqref>
+          <xm:sqref>BP3:BP1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4CA88649-FA21-4E18-8525-72E3D0112FE0}">
           <x14:formula1>
             <xm:f>Hoja2!$AA$2:$AA$126</xm:f>
           </x14:formula1>
-          <xm:sqref>BT3:BT1048576 BU3:BU1048576 BV3:BV1048576</xm:sqref>
+          <xm:sqref>BU3:BU1048576 BV3:BV1048576 BW3:BW1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3172409-A8B4-45E9-A35A-A489AFE1480C}">
           <x14:formula1>
             <xm:f>Hoja2!$AB$2:$AB$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BW3:BW1048576</xm:sqref>
+          <xm:sqref>BX3:BX1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Fix ficha tecnica, fix trait
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sgc\storage\app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00B4514-750A-4432-A8C9-C3136E81B986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1269F4-E27E-4485-B3B0-B6D714F49069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{28BFEBC5-EF34-42C7-846D-BB644F26337B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="419">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -1289,6 +1289,9 @@
   </si>
   <si>
     <t>PROPIETARIO</t>
+  </si>
+  <si>
+    <t>razon social</t>
   </si>
 </sst>
 </file>
@@ -1726,7 +1729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7806A9-AE76-44CF-993F-CC0D365B724C}">
-  <dimension ref="A1:CF5"/>
+  <dimension ref="A1:CG5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -1743,47 +1746,47 @@
     <col min="12" max="12" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.88671875" customWidth="1"/>
-    <col min="23" max="23" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="20.88671875" style="7" customWidth="1"/>
-    <col min="42" max="42" width="16" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="26" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="51" max="52" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="11.5546875" style="7"/>
-    <col min="70" max="70" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="20.109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="16" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="31" customWidth="1"/>
+    <col min="19" max="19" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.88671875" customWidth="1"/>
+    <col min="24" max="24" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="20.88671875" style="7" customWidth="1"/>
+    <col min="43" max="43" width="16" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="26" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="11.5546875" style="7"/>
+    <col min="71" max="71" width="13.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="14.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="20.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="16" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:85" s="3" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1811,10 +1814,10 @@
       <c r="S1" s="10"/>
       <c r="T1" s="10"/>
       <c r="U1" s="10"/>
-      <c r="V1" s="11" t="s">
+      <c r="V1" s="10"/>
+      <c r="W1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="W1" s="11"/>
       <c r="X1" s="11"/>
       <c r="Y1" s="11"/>
       <c r="Z1" s="11"/>
@@ -1832,13 +1835,13 @@
       <c r="AL1" s="11"/>
       <c r="AM1" s="11"/>
       <c r="AN1" s="11"/>
-      <c r="AO1" s="1" t="s">
+      <c r="AO1" s="11"/>
+      <c r="AP1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AP1" s="12" t="s">
+      <c r="AQ1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="AQ1" s="12"/>
       <c r="AR1" s="12"/>
       <c r="AS1" s="12"/>
       <c r="AT1" s="12"/>
@@ -1864,30 +1867,31 @@
       <c r="BN1" s="12"/>
       <c r="BO1" s="12"/>
       <c r="BP1" s="12"/>
-      <c r="BQ1" s="10" t="s">
+      <c r="BQ1" s="12"/>
+      <c r="BR1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="BR1" s="10"/>
       <c r="BS1" s="10"/>
       <c r="BT1" s="10"/>
       <c r="BU1" s="10"/>
       <c r="BV1" s="10"/>
       <c r="BW1" s="10"/>
       <c r="BX1" s="10"/>
-      <c r="BY1" s="8" t="s">
+      <c r="BY1" s="10"/>
+      <c r="BZ1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="BZ1" s="8"/>
       <c r="CA1" s="8"/>
       <c r="CB1" s="8"/>
       <c r="CC1" s="8"/>
       <c r="CD1" s="8"/>
       <c r="CE1" s="8"/>
-      <c r="CF1" s="2" t="s">
+      <c r="CF1" s="8"/>
+      <c r="CG1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:84" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:85" s="6" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -1940,228 +1944,231 @@
         <v>23</v>
       </c>
       <c r="R2" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AO2" s="5" t="s">
+      <c r="AP2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="AW2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="BO2" s="4" t="s">
+      <c r="BP2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="BP2" s="4" t="s">
+      <c r="BQ2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="BQ2" s="5" t="s">
+      <c r="BR2" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="BR2" s="5" t="s">
+      <c r="BS2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="BS2" s="5" t="s">
+      <c r="BT2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="BT2" s="5" t="s">
+      <c r="BU2" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="BU2" s="4" t="s">
+      <c r="BV2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="BV2" s="4" t="s">
+      <c r="BW2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="BW2" s="4" t="s">
+      <c r="BX2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="BX2" s="4" t="s">
+      <c r="BY2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="BY2" s="4" t="s">
+      <c r="BZ2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="BZ2" s="4" t="s">
+      <c r="CA2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="CA2" s="4" t="s">
+      <c r="CB2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="CB2" s="4" t="s">
+      <c r="CC2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="CC2" s="4" t="s">
+      <c r="CD2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="CD2" s="4" t="s">
+      <c r="CE2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="CE2" s="4" t="s">
+      <c r="CF2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="CF2" s="4" t="s">
+      <c r="CG2" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="BU3" s="7"/>
-      <c r="BX3" s="7"/>
-    </row>
-    <row r="4" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="BU4" s="7"/>
-      <c r="BX4" s="7"/>
-    </row>
-    <row r="5" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="BU5" s="7"/>
-      <c r="BX5" s="7"/>
+    <row r="3" spans="1:85" x14ac:dyDescent="0.3">
+      <c r="BV3" s="7"/>
+      <c r="BY3" s="7"/>
+    </row>
+    <row r="4" spans="1:85" x14ac:dyDescent="0.3">
+      <c r="BV4" s="7"/>
+      <c r="BY4" s="7"/>
+    </row>
+    <row r="5" spans="1:85" x14ac:dyDescent="0.3">
+      <c r="BV5" s="7"/>
+      <c r="BY5" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="BY1:CE1"/>
+    <mergeCell ref="BZ1:CF1"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:N1"/>
-    <mergeCell ref="O1:U1"/>
-    <mergeCell ref="V1:AN1"/>
-    <mergeCell ref="AP1:BP1"/>
-    <mergeCell ref="BQ1:BX1"/>
+    <mergeCell ref="O1:V1"/>
+    <mergeCell ref="W1:AO1"/>
+    <mergeCell ref="AQ1:BQ1"/>
+    <mergeCell ref="BR1:BY1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2172,7 +2179,7 @@
           <x14:formula1>
             <xm:f>Hoja2!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>R3:R1048576</xm:sqref>
+          <xm:sqref>S3:S1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E50DB94-E1AA-4CE4-ADEF-83A1F4AB5B43}">
           <x14:formula1>
@@ -2184,163 +2191,163 @@
           <x14:formula1>
             <xm:f>Hoja2!$B$2:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>S3:S1048576</xm:sqref>
+          <xm:sqref>T3:T1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E07B1B75-AF03-4A8D-BC24-5721557FF61A}">
           <x14:formula1>
             <xm:f>Hoja2!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>U3:U1048576 AR3:AR1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576 AV3:AV1048576 AW3:AW1048576</xm:sqref>
+          <xm:sqref>V3:V1048576 AS3:AS1048576 AT3:AT1048576 AU3:AU1048576 AV3:AV1048576 AW3:AW1048576 AX3:AX1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{41BB7C65-DC93-4292-81A0-F268D8A02A18}">
           <x14:formula1>
             <xm:f>Hoja2!$D$2:$D$45</xm:f>
           </x14:formula1>
-          <xm:sqref>V3:V1048576</xm:sqref>
+          <xm:sqref>W3:W1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D9C52FE-6D55-407E-8C4B-88B2DEF94573}">
           <x14:formula1>
             <xm:f>Hoja2!$E$2:$E$31</xm:f>
           </x14:formula1>
-          <xm:sqref>X3:X1048576</xm:sqref>
+          <xm:sqref>Y3:Y1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{84E5F63A-A4AB-47B5-97BA-AA3C8554A144}">
           <x14:formula1>
             <xm:f>Hoja2!$F$2:$F$26</xm:f>
           </x14:formula1>
-          <xm:sqref>AP3:AP1048576</xm:sqref>
+          <xm:sqref>AQ3:AQ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7D33DAEA-F9F3-4874-B861-42A021DC99B1}">
           <x14:formula1>
             <xm:f>Hoja2!$H$2:$H$6</xm:f>
           </x14:formula1>
-          <xm:sqref>AX3:AX1048576</xm:sqref>
+          <xm:sqref>AY3:AY1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{161264C7-A5E3-4F61-A614-028D62F3EC0E}">
           <x14:formula1>
             <xm:f>Hoja2!$I$2:$I$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AY3:AY1048576</xm:sqref>
+          <xm:sqref>AZ3:AZ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{795EBF0F-0DAD-4EB9-A428-BD50873910D0}">
           <x14:formula1>
             <xm:f>Hoja2!$J$2:$J$8</xm:f>
           </x14:formula1>
-          <xm:sqref>AZ3:AZ1048576</xm:sqref>
+          <xm:sqref>BA3:BA1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{28A1E571-1CEC-47BF-825E-67A9E930A0D3}">
           <x14:formula1>
             <xm:f>Hoja2!$K$2:$K$11</xm:f>
           </x14:formula1>
-          <xm:sqref>BA3:BA1048576</xm:sqref>
+          <xm:sqref>BB3:BB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F2DCA628-14C7-4F71-A7C2-378A86B56965}">
           <x14:formula1>
             <xm:f>Hoja2!$L$2:$L$8</xm:f>
           </x14:formula1>
-          <xm:sqref>BB3:BB1048576</xm:sqref>
+          <xm:sqref>BC3:BC1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25227AEB-E170-440B-A489-C54B8AAA71EE}">
           <x14:formula1>
             <xm:f>Hoja2!$M$2:$M$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BC3:BC1048576</xm:sqref>
+          <xm:sqref>BD3:BD1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{14392394-449F-4C32-B560-7CCB1753B746}">
           <x14:formula1>
             <xm:f>Hoja2!$N$2:$N$8</xm:f>
           </x14:formula1>
-          <xm:sqref>BD3:BD1048576</xm:sqref>
+          <xm:sqref>BE3:BE1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7144E9CC-E537-4DC0-B364-139231DFAEF2}">
           <x14:formula1>
             <xm:f>Hoja2!$O$2:$O$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BE3:BE1048576</xm:sqref>
+          <xm:sqref>BF3:BF1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{22524E45-CF71-4F27-95AC-5851CBA321A6}">
           <x14:formula1>
             <xm:f>Hoja2!$P$2:$P$9</xm:f>
           </x14:formula1>
-          <xm:sqref>BF3:BF1048576</xm:sqref>
+          <xm:sqref>BG3:BG1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{46DF2204-513F-4B04-B29F-399B0D420994}">
           <x14:formula1>
             <xm:f>Hoja2!$Q$2:$Q$6</xm:f>
           </x14:formula1>
-          <xm:sqref>BG3:BG1048576</xm:sqref>
+          <xm:sqref>BH3:BH1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{66E24F7D-787B-4D0F-85D0-6816BB1C4822}">
           <x14:formula1>
             <xm:f>Hoja2!$R$2:$R$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BH3:BH1048576</xm:sqref>
+          <xm:sqref>BI3:BI1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5F22308-7CEA-4033-995C-256C6A7FAD4A}">
           <x14:formula1>
             <xm:f>Hoja2!$S$2:$S$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BI3:BI1048576</xm:sqref>
+          <xm:sqref>BJ3:BJ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{048FD807-791D-4C41-9CAE-8C262B2803EA}">
           <x14:formula1>
             <xm:f>Hoja2!$T$2:$T$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BJ3:BJ1048576</xm:sqref>
+          <xm:sqref>BK3:BK1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7CA12FC9-A5C1-479E-B2EE-19C704ABBAB2}">
           <x14:formula1>
             <xm:f>Hoja2!$U$2:$U$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BK3:BK1048576</xm:sqref>
+          <xm:sqref>BL3:BL1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E3AB702-C42C-4122-9A12-001CB2150602}">
           <x14:formula1>
             <xm:f>Hoja2!$V$2:$V$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BL3:BL1048576</xm:sqref>
+          <xm:sqref>BM3:BM1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9BC56ED0-C878-4B70-AF59-878EF8AA865E}">
           <x14:formula1>
             <xm:f>Hoja2!$W$2:$W$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BM3:BM1048576</xm:sqref>
+          <xm:sqref>BN3:BN1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0E1A2C55-058E-4225-A3E9-B4F625D85399}">
           <x14:formula1>
             <xm:f>Hoja2!$X$2:$X$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BN3:BN1048576</xm:sqref>
+          <xm:sqref>BO3:BO1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7BF7C810-BC07-467A-B909-741F16C106B4}">
           <x14:formula1>
             <xm:f>Hoja2!$Y$2:$Y$4</xm:f>
           </x14:formula1>
-          <xm:sqref>BO3:BO1048576</xm:sqref>
+          <xm:sqref>BP3:BP1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{60069B37-3CC2-4FE5-ABC6-4FCA59061E75}">
           <x14:formula1>
             <xm:f>Hoja2!$Z$2:$Z$5</xm:f>
           </x14:formula1>
-          <xm:sqref>BP3:BP1048576</xm:sqref>
+          <xm:sqref>BQ3:BQ1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4CA88649-FA21-4E18-8525-72E3D0112FE0}">
           <x14:formula1>
             <xm:f>Hoja2!$AA$2:$AA$126</xm:f>
           </x14:formula1>
-          <xm:sqref>BU3:BU1048576 BV3:BV1048576 BW3:BW1048576</xm:sqref>
+          <xm:sqref>BV3:BV1048576 BW3:BW1048576 BX3:BX1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B3172409-A8B4-45E9-A35A-A489AFE1480C}">
           <x14:formula1>
             <xm:f>Hoja2!$AB$2:$AB$7</xm:f>
           </x14:formula1>
-          <xm:sqref>BX3:BX1048576</xm:sqref>
+          <xm:sqref>BY3:BY1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2AF1B496-69B3-4CB2-9F04-1DACE3D47967}">
           <x14:formula1>
             <xm:f>Hoja2!$G$2:$G$12</xm:f>
           </x14:formula1>
-          <xm:sqref>AQ1:AQ1048576</xm:sqref>
+          <xm:sqref>AR1:AR1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se finalizo ficha tecnica simple, se agrego funcion para generar tramites de certificados mediante jobs
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ODS\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ODS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2464676C-208B-4145-A025-D0E737632637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EECF47-8BE7-486C-B7AD-CDBB577681E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8A8D1F3A-9481-47DB-BED2-2431B12C011C}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{8A8D1F3A-9481-47DB-BED2-2431B12C011C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -976,9 +976,6 @@
     <t>uso construccion</t>
   </si>
   <si>
-    <t>estado construccion</t>
-  </si>
-  <si>
     <t>calidad construccion</t>
   </si>
   <si>
@@ -1013,6 +1010,9 @@
   </si>
   <si>
     <t>agua potable</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> estado construccion</t>
   </si>
 </sst>
 </file>
@@ -1497,55 +1497,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CC64A88-BD29-458A-8144-6183040809A8}">
   <dimension ref="A1:BN13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="14" max="14" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.69140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.3828125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.84375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.3828125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.53515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.15234375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.15234375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.53515625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.69140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.15234375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.3828125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.53515625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.15234375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.69140625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="21" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="25.3046875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="17.15234375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20.15234375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="16.3828125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.15234375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.84375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="16.3046875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.69140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="18.69140625" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="19" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="52" max="54" width="11.42578125" style="10"/>
-    <col min="55" max="55" width="26.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="26.7109375" style="10" customWidth="1"/>
-    <col min="58" max="58" width="12.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="10.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="15.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="17.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="9.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="54.28515625" customWidth="1"/>
-    <col min="65" max="65" width="44.5703125" customWidth="1"/>
-    <col min="66" max="66" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="11.42578125" customWidth="1"/>
+    <col min="44" max="44" width="7.3828125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="28.3046875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.69140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="54" width="11.3828125" style="10"/>
+    <col min="55" max="55" width="26.69140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="56" max="57" width="26.69140625" style="10" customWidth="1"/>
+    <col min="58" max="58" width="12.3828125" style="10" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="7.84375" style="10" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="10.53515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="15.69140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="17.69140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="9.3828125" style="10" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="54.3046875" customWidth="1"/>
+    <col min="65" max="65" width="44.53515625" customWidth="1"/>
+    <col min="66" max="66" width="22.3828125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:66" ht="18.45" x14ac:dyDescent="0.4">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1633,7 +1633,7 @@
       <c r="BM1" s="5"/>
       <c r="BN1" s="2"/>
     </row>
-    <row r="2" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -1641,13 +1641,13 @@
         <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>13</v>
@@ -1761,16 +1761,16 @@
         <v>312</v>
       </c>
       <c r="AQ2" s="3" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="AR2" s="3" t="s">
         <v>45</v>
       </c>
       <c r="AS2" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AT2" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="AT2" s="3" t="s">
-        <v>315</v>
       </c>
       <c r="AU2" s="3" t="s">
         <v>308</v>
@@ -1782,10 +1782,10 @@
         <v>43</v>
       </c>
       <c r="AX2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AY2" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="AY2" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="AZ2" s="11" t="s">
         <v>300</v>
@@ -1803,25 +1803,25 @@
         <v>296</v>
       </c>
       <c r="BE2" s="11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="BF2" s="11" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="BG2" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="BH2" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="BH2" s="11" t="s">
+      <c r="BI2" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="BI2" s="11" t="s">
+      <c r="BJ2" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="BJ2" s="11" t="s">
+      <c r="BK2" s="11" t="s">
         <v>322</v>
-      </c>
-      <c r="BK2" s="11" t="s">
-        <v>323</v>
       </c>
       <c r="BL2" s="3" t="s">
         <v>46</v>
@@ -1833,10 +1833,10 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:66" x14ac:dyDescent="0.4">
       <c r="D3" s="10"/>
     </row>
-    <row r="4" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -1892,7 +1892,7 @@
       <c r="BM4" s="10"/>
       <c r="BN4" s="10"/>
     </row>
-    <row r="5" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -1948,7 +1948,7 @@
       <c r="BM5" s="10"/>
       <c r="BN5" s="10"/>
     </row>
-    <row r="6" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2004,7 +2004,7 @@
       <c r="BM6" s="10"/>
       <c r="BN6" s="10"/>
     </row>
-    <row r="7" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -2060,7 +2060,7 @@
       <c r="BM7" s="10"/>
       <c r="BN7" s="10"/>
     </row>
-    <row r="8" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -2116,7 +2116,7 @@
       <c r="BM8" s="10"/>
       <c r="BN8" s="10"/>
     </row>
-    <row r="9" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -2172,7 +2172,7 @@
       <c r="BM9" s="10"/>
       <c r="BN9" s="10"/>
     </row>
-    <row r="10" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2228,7 +2228,7 @@
       <c r="BM10" s="10"/>
       <c r="BN10" s="10"/>
     </row>
-    <row r="11" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2284,7 +2284,7 @@
       <c r="BM11" s="10"/>
       <c r="BN11" s="10"/>
     </row>
-    <row r="12" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2340,7 +2340,7 @@
       <c r="BM12" s="10"/>
       <c r="BN12" s="10"/>
     </row>
-    <row r="13" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:66" x14ac:dyDescent="0.4">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2470,20 +2470,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF097C49-C947-4EF3-9D3B-516C3E7919D3}">
   <dimension ref="A1:J126"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.84375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.15234375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="40.84375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>298</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>293</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>286</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B4" s="7" t="s">
         <v>277</v>
       </c>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B5" s="7" t="s">
         <v>270</v>
       </c>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B6" s="7" t="s">
         <v>263</v>
       </c>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B7" s="7" t="s">
         <v>256</v>
       </c>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C8" s="8" t="s">
         <v>249</v>
       </c>
@@ -2694,7 +2694,7 @@
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C9" s="8" t="s">
         <v>244</v>
       </c>
@@ -2713,7 +2713,7 @@
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C10" s="8" t="s">
         <v>239</v>
       </c>
@@ -2732,7 +2732,7 @@
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C11" s="8" t="s">
         <v>234</v>
       </c>
@@ -2751,7 +2751,7 @@
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C12" s="8" t="s">
         <v>229</v>
       </c>
@@ -2770,7 +2770,7 @@
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C13" s="8" t="s">
         <v>201</v>
       </c>
@@ -2789,7 +2789,7 @@
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C14" s="8" t="s">
         <v>221</v>
       </c>
@@ -2806,7 +2806,7 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C15" s="8" t="s">
         <v>217</v>
       </c>
@@ -2823,7 +2823,7 @@
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="C16" s="8" t="s">
         <v>213</v>
       </c>
@@ -2840,7 +2840,7 @@
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C17" s="8" t="s">
         <v>209</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C18" s="8" t="s">
         <v>206</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C19" s="8" t="s">
         <v>202</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C20" s="8" t="s">
         <v>198</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C21" s="8" t="s">
         <v>194</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C22" s="8" t="s">
         <v>190</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C23" s="8" t="s">
         <v>186</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C24" s="8" t="s">
         <v>182</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C25" s="8" t="s">
         <v>178</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C26" s="8" t="s">
         <v>171</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C27" s="8" t="s">
         <v>168</v>
       </c>
@@ -3003,7 +3003,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C28" s="8" t="s">
         <v>169</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C29" s="8" t="s">
         <v>166</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C30" s="8" t="s">
         <v>163</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C31" s="8" t="s">
         <v>161</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C32" s="8" t="s">
         <v>158</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C33" s="8" t="s">
         <v>156</v>
       </c>
@@ -3075,7 +3075,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C34" s="8" t="s">
         <v>154</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C35" s="8" t="s">
         <v>152</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C36" s="8" t="s">
         <v>150</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C37" s="8" t="s">
         <v>148</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C38" s="8" t="s">
         <v>146</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C39" s="8" t="s">
         <v>144</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C40" s="8" t="s">
         <v>142</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C41" s="8" t="s">
         <v>140</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C42" s="8" t="s">
         <v>138</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C43" s="8" t="s">
         <v>136</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C44" s="8" t="s">
         <v>134</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:7" x14ac:dyDescent="0.4">
       <c r="C45" s="8" t="s">
         <v>132</v>
       </c>
@@ -3195,413 +3195,413 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:7" x14ac:dyDescent="0.4">
       <c r="E46" s="10"/>
       <c r="F46" s="10"/>
       <c r="G46" s="10" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:7" x14ac:dyDescent="0.4">
       <c r="E47" s="10"/>
       <c r="F47" s="10"/>
       <c r="G47" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:7" x14ac:dyDescent="0.4">
       <c r="E48" s="10"/>
       <c r="F48" s="10"/>
       <c r="G48" s="10" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G49" s="10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G50" s="10" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G51" s="10" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G52" s="10" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="53" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G53" s="10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="54" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G54" s="10" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="55" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G55" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="56" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G56" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="57" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G57" s="10" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G58" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="59" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G59" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G60" s="10" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G61" s="10" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="62" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G62" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="63" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G63" s="10" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="64" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G64" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="65" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G65" s="10" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="66" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G66" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="67" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G67" s="10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="68" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G68" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="69" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G69" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="70" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G70" s="10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="71" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G71" s="10" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="72" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G72" s="10" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="73" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G73" s="10" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="74" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G74" s="10" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="75" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G75" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="76" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G76" s="10" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G77" s="10" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="78" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G78" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="79" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G79" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G80" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="81" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G81" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="82" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G82" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="83" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G83" s="10" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="84" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G84" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G85" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="86" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G86" s="10" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="87" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G87" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="88" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G88" s="10" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="89" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G89" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G90" s="10" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="91" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G91" s="10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="92" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G92" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="93" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G93" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="94" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G94" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="95" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G95" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="96" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G96" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="97" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G97" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="98" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G98" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="99" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G99" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="100" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G100" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="101" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G101" s="10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="102" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G102" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="103" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G103" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="104" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G104" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="105" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G105" s="10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="106" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G106" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="107" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G107" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="108" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G108" s="10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="109" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G109" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="110" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G110" s="10" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="111" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G111" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G112" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="113" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G113" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="114" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G114" s="10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="115" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G115" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="116" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G116" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="117" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G117" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="118" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G118" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="119" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G119" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="120" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G120" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="121" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G121" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="122" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G122" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="123" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G123" s="10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="124" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G124" s="10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="125" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G125" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="126" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G126" s="10" t="s">
         <v>50</v>
       </c>

</xml_diff>

<commit_message>
Se agrego predio origen a ficha tecnica, se agrego funcion para ignorar filas que no contienen cuenta predial en ficha tecnica
</commit_message>
<xml_diff>
--- a/storage/app/public/ficha_tecnica.xlsx
+++ b/storage/app/public/ficha_tecnica.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ODS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EECF47-8BE7-486C-B7AD-CDBB577681E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE6BA1D-0340-4652-A8D6-C3A3477A06CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{8A8D1F3A-9481-47DB-BED2-2431B12C011C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8A8D1F3A-9481-47DB-BED2-2431B12C011C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="326">
   <si>
     <t>Cuenta Predial</t>
   </si>
@@ -1013,6 +1013,9 @@
   </si>
   <si>
     <t xml:space="preserve"> estado construccion</t>
+  </si>
+  <si>
+    <t>predio origen</t>
   </si>
 </sst>
 </file>
@@ -1496,56 +1499,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CC64A88-BD29-458A-8144-6183040809A8}">
-  <dimension ref="A1:BN13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:BO13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="14" max="14" width="13.69140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.3828125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.84375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.3828125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.53515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.15234375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.15234375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.53515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.69140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.15234375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.3828125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="17.53515625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.15234375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.69140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="21" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="25.3046875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.15234375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="20.15234375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.15234375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.84375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="16.3046875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.69140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="18.69140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="19" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="7.3828125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="28.3046875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.69140625" bestFit="1" customWidth="1"/>
-    <col min="52" max="54" width="11.3828125" style="10"/>
-    <col min="55" max="55" width="26.69140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="26.69140625" style="10" customWidth="1"/>
-    <col min="58" max="58" width="12.3828125" style="10" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.84375" style="10" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="10.53515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="15.69140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="17.69140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="9.3828125" style="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="54.3046875" customWidth="1"/>
-    <col min="65" max="65" width="44.53515625" customWidth="1"/>
-    <col min="66" max="66" width="22.3828125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="11.3828125" customWidth="1"/>
+    <col min="44" max="44" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="52" max="54" width="11.42578125" style="10"/>
+    <col min="55" max="55" width="26.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="56" max="57" width="26.7109375" style="10" customWidth="1"/>
+    <col min="58" max="58" width="12.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="7.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="10.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="15.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="17.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="9.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="54.28515625" customWidth="1"/>
+    <col min="65" max="65" width="44.5703125" customWidth="1"/>
+    <col min="66" max="66" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="18.45" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:67" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1632,8 +1635,9 @@
       </c>
       <c r="BM1" s="5"/>
       <c r="BN1" s="2"/>
-    </row>
-    <row r="2" spans="1:66" x14ac:dyDescent="0.4">
+      <c r="BO1" s="2"/>
+    </row>
+    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -1832,11 +1836,14 @@
       <c r="BN2" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="3" spans="1:66" x14ac:dyDescent="0.4">
+      <c r="BO2" s="11" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
       <c r="D3" s="10"/>
     </row>
-    <row r="4" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -1892,7 +1899,7 @@
       <c r="BM4" s="10"/>
       <c r="BN4" s="10"/>
     </row>
-    <row r="5" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -1948,7 +1955,7 @@
       <c r="BM5" s="10"/>
       <c r="BN5" s="10"/>
     </row>
-    <row r="6" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2004,7 +2011,7 @@
       <c r="BM6" s="10"/>
       <c r="BN6" s="10"/>
     </row>
-    <row r="7" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -2060,7 +2067,7 @@
       <c r="BM7" s="10"/>
       <c r="BN7" s="10"/>
     </row>
-    <row r="8" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -2116,7 +2123,7 @@
       <c r="BM8" s="10"/>
       <c r="BN8" s="10"/>
     </row>
-    <row r="9" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -2172,7 +2179,7 @@
       <c r="BM9" s="10"/>
       <c r="BN9" s="10"/>
     </row>
-    <row r="10" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2228,7 +2235,7 @@
       <c r="BM10" s="10"/>
       <c r="BN10" s="10"/>
     </row>
-    <row r="11" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2284,7 +2291,7 @@
       <c r="BM11" s="10"/>
       <c r="BN11" s="10"/>
     </row>
-    <row r="12" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2340,7 +2347,7 @@
       <c r="BM12" s="10"/>
       <c r="BN12" s="10"/>
     </row>
-    <row r="13" spans="1:66" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2435,7 +2442,7 @@
           <x14:formula1>
             <xm:f>Hoja4!$J$2:$J$3</xm:f>
           </x14:formula1>
-          <xm:sqref>BN3:BN1048576 BF3:BK1048576</xm:sqref>
+          <xm:sqref>BN3:BN1048576 BF3:BK1048576 BO3:BO1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B04FBD7A-2648-450E-BD58-F72C45772D32}">
           <x14:formula1>
@@ -2470,20 +2477,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF097C49-C947-4EF3-9D3B-516C3E7919D3}">
   <dimension ref="A1:J126"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.15234375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.84375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.84375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40.84375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.53515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>298</v>
       </c>
@@ -2515,7 +2522,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>293</v>
       </c>
@@ -2547,7 +2554,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>286</v>
       </c>
@@ -2579,7 +2586,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>277</v>
       </c>
@@ -2603,7 +2610,7 @@
       </c>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
         <v>270</v>
       </c>
@@ -2627,7 +2634,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
         <v>263</v>
       </c>
@@ -2651,7 +2658,7 @@
       </c>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>256</v>
       </c>
@@ -2675,7 +2682,7 @@
       </c>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C8" s="8" t="s">
         <v>249</v>
       </c>
@@ -2694,7 +2701,7 @@
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" s="8" t="s">
         <v>244</v>
       </c>
@@ -2713,7 +2720,7 @@
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" s="8" t="s">
         <v>239</v>
       </c>
@@ -2732,7 +2739,7 @@
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C11" s="8" t="s">
         <v>234</v>
       </c>
@@ -2751,7 +2758,7 @@
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" s="8" t="s">
         <v>229</v>
       </c>
@@ -2770,7 +2777,7 @@
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C13" s="8" t="s">
         <v>201</v>
       </c>
@@ -2789,7 +2796,7 @@
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C14" s="8" t="s">
         <v>221</v>
       </c>
@@ -2806,7 +2813,7 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C15" s="8" t="s">
         <v>217</v>
       </c>
@@ -2823,7 +2830,7 @@
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C16" s="8" t="s">
         <v>213</v>
       </c>
@@ -2840,7 +2847,7 @@
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C17" s="8" t="s">
         <v>209</v>
       </c>
@@ -2855,7 +2862,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C18" s="8" t="s">
         <v>206</v>
       </c>
@@ -2870,7 +2877,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C19" s="8" t="s">
         <v>202</v>
       </c>
@@ -2885,7 +2892,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C20" s="8" t="s">
         <v>198</v>
       </c>
@@ -2900,7 +2907,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C21" s="8" t="s">
         <v>194</v>
       </c>
@@ -2915,7 +2922,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C22" s="8" t="s">
         <v>190</v>
       </c>
@@ -2930,7 +2937,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C23" s="8" t="s">
         <v>186</v>
       </c>
@@ -2945,7 +2952,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C24" s="8" t="s">
         <v>182</v>
       </c>
@@ -2960,7 +2967,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C25" s="8" t="s">
         <v>178</v>
       </c>
@@ -2975,7 +2982,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C26" s="8" t="s">
         <v>171</v>
       </c>
@@ -2990,7 +2997,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C27" s="8" t="s">
         <v>168</v>
       </c>
@@ -3003,7 +3010,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C28" s="8" t="s">
         <v>169</v>
       </c>
@@ -3016,7 +3023,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C29" s="8" t="s">
         <v>166</v>
       </c>
@@ -3029,7 +3036,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C30" s="8" t="s">
         <v>163</v>
       </c>
@@ -3042,7 +3049,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C31" s="8" t="s">
         <v>161</v>
       </c>
@@ -3055,7 +3062,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C32" s="8" t="s">
         <v>158</v>
       </c>
@@ -3065,7 +3072,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C33" s="8" t="s">
         <v>156</v>
       </c>
@@ -3075,7 +3082,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C34" s="8" t="s">
         <v>154</v>
       </c>
@@ -3085,7 +3092,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C35" s="8" t="s">
         <v>152</v>
       </c>
@@ -3095,7 +3102,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C36" s="8" t="s">
         <v>150</v>
       </c>
@@ -3105,7 +3112,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C37" s="8" t="s">
         <v>148</v>
       </c>
@@ -3115,7 +3122,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C38" s="8" t="s">
         <v>146</v>
       </c>
@@ -3125,7 +3132,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C39" s="8" t="s">
         <v>144</v>
       </c>
@@ -3135,7 +3142,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C40" s="8" t="s">
         <v>142</v>
       </c>
@@ -3145,7 +3152,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C41" s="8" t="s">
         <v>140</v>
       </c>
@@ -3155,7 +3162,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C42" s="8" t="s">
         <v>138</v>
       </c>
@@ -3165,7 +3172,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C43" s="8" t="s">
         <v>136</v>
       </c>
@@ -3175,7 +3182,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C44" s="8" t="s">
         <v>134</v>
       </c>
@@ -3185,7 +3192,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C45" s="8" t="s">
         <v>132</v>
       </c>
@@ -3195,413 +3202,413 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
       <c r="E46" s="10"/>
       <c r="F46" s="10"/>
       <c r="G46" s="10" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
       <c r="E47" s="10"/>
       <c r="F47" s="10"/>
       <c r="G47" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
       <c r="E48" s="10"/>
       <c r="F48" s="10"/>
       <c r="G48" s="10" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="49" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="50" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G50" s="10" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G51" s="10" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="52" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G52" s="10" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="53" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="53" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G53" s="10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="54" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="54" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G54" s="10" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="55" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="55" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G55" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="56" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="56" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G56" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="57" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="57" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G57" s="10" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="58" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G58" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="59" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="59" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G59" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="60" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G60" s="10" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="61" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G61" s="10" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="62" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="62" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G62" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="63" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="63" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G63" s="10" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="64" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="64" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G64" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="65" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="65" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G65" s="10" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="66" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="66" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G66" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="67" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="67" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G67" s="10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="68" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="68" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G68" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="69" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="69" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G69" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="70" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="70" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G70" s="10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="71" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="71" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G71" s="10" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="72" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="72" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G72" s="10" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="73" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="73" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G73" s="10" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="74" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="74" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G74" s="10" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="75" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="75" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G75" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="76" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="76" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G76" s="10" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="77" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G77" s="10" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="78" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="78" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G78" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="79" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="79" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G79" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="80" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G80" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="81" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="81" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G81" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="82" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="82" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G82" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="83" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="83" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G83" s="10" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="84" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="84" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G84" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="85" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G85" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="86" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="86" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G86" s="10" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="87" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="87" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G87" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="88" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="88" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G88" s="10" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="89" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="89" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G89" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="90" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G90" s="10" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="91" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="91" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G91" s="10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="92" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="92" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G92" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="93" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="93" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G93" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="94" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="94" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G94" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="95" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="95" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G95" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="96" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="96" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G96" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="97" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="97" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G97" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="98" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="98" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G98" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="99" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="99" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G99" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="100" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="100" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G100" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="101" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="101" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G101" s="10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="102" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="102" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G102" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="103" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="103" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G103" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="104" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="104" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G104" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="105" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="105" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G105" s="10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="106" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="106" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G106" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="107" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="107" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G107" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="108" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="108" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G108" s="10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="109" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="109" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G109" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="110" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="110" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G110" s="10" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="111" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="111" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G111" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="112" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G112" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="113" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="113" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G113" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="114" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="114" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G114" s="10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="115" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="115" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G115" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="116" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="116" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G116" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="117" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="117" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G117" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="118" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="118" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G118" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="119" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="119" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G119" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="120" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="120" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G120" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="121" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="121" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G121" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="122" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="122" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G122" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="123" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="123" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G123" s="10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="124" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="124" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G124" s="10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="125" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="125" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G125" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="126" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="126" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G126" s="10" t="s">
         <v>50</v>
       </c>

</xml_diff>